<commit_message>
feat(radio): measure masters and resolve cue reachability
</commit_message>
<xml_diff>
--- a/docs/audits/SQUATCHSMASH-RADIO-AUDIT.xlsx
+++ b/docs/audits/SQUATCHSMASH-RADIO-AUDIT.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scene Timeline" sheetId="1" r:id="R2f06da62845a4fe4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Station Catalog" sheetId="2" r:id="Rb33bb42d8bb749a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cue Inventory" sheetId="3" r:id="R97f05b39ca8943d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Problems and Decisions" sheetId="4" r:id="Rb5420ad86d4f4a0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revamp Plan" sheetId="5" r:id="R767fd1cdf5ef4e68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scene Timeline" sheetId="1" r:id="Re97fc961620f4b0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Station Catalog" sheetId="2" r:id="R13e72fa051ce4744"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cue Inventory" sheetId="3" r:id="R7ff68e4b5cb54587"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Problems and Decisions" sheetId="4" r:id="R652078f99ae04668"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revamp Plan" sheetId="5" r:id="Rc93aad9db3204e1f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4008,7 +4008,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf22089f8a4c04289"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51349b543a82474a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4255,7 +4255,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd768c902d9be4800"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77ec43683e3741dd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4413,13 +4413,13 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L6" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Measured: -13.69 LUFS integrated; 0.08 dBTP 4× estimate; 0.08 dBFS sample peak</x:v>
       </x:c>
       <x:c r="M6" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
       </x:c>
       <x:c r="N6" s="21" t="str">
-        <x:v>Keep; verify audible content and loudness in the active scene.</x:v>
+        <x:v>Keep; loudness is hash-bound. Verify audible content, dialogue masking, and lifecycle in the active scene.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="46" customHeight="1">
@@ -4457,13 +4457,13 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L7" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Measured: -14.07 LUFS integrated; -0.06 dBTP 4× estimate; -0.09 dBFS sample peak</x:v>
       </x:c>
       <x:c r="M7" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
       </x:c>
       <x:c r="N7" s="21" t="str">
-        <x:v>Keep; verify audible content and loudness in the active scene.</x:v>
+        <x:v>Keep; loudness is hash-bound. Verify audible content, dialogue masking, and lifecycle in the active scene.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="46" customHeight="1">
@@ -4501,13 +4501,13 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L8" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Measured: -16.04 LUFS integrated; -5.79 dBTP 4× estimate; -5.92 dBFS sample peak</x:v>
       </x:c>
       <x:c r="M8" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
       </x:c>
       <x:c r="N8" s="21" t="str">
-        <x:v>Keep; verify audible content and loudness in the active scene.</x:v>
+        <x:v>Keep; loudness is hash-bound. Verify audible content, dialogue masking, and lifecycle in the active scene.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="46" customHeight="1">
@@ -4545,13 +4545,13 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L9" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Measured: -12.09 LUFS integrated; -0.45 dBTP 4× estimate; -0.45 dBFS sample peak</x:v>
       </x:c>
       <x:c r="M9" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
       </x:c>
       <x:c r="N9" s="21" t="str">
-        <x:v>Keep; verify audible content and loudness in the active scene.</x:v>
+        <x:v>Keep; loudness is hash-bound. Verify audible content, dialogue masking, and lifecycle in the active scene.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="46" customHeight="1">
@@ -4589,13 +4589,13 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L10" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Measured: -12.2 LUFS integrated; -1.14 dBTP 4× estimate; -1.14 dBFS sample peak</x:v>
       </x:c>
       <x:c r="M10" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
       </x:c>
       <x:c r="N10" s="21" t="str">
-        <x:v>Keep; verify audible content and loudness in the active scene.</x:v>
+        <x:v>Keep; loudness is hash-bound. Verify audible content, dialogue masking, and lifecycle in the active scene.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="46" customHeight="1">
@@ -4633,13 +4633,13 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L11" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Measured: -12.58 LUFS integrated; -0.95 dBTP 4× estimate; -1.08 dBFS sample peak</x:v>
       </x:c>
       <x:c r="M11" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
       </x:c>
       <x:c r="N11" s="21" t="str">
-        <x:v>Keep; verify audible content and loudness in the active scene.</x:v>
+        <x:v>Keep; loudness is hash-bound. Verify audible content, dialogue masking, and lifecycle in the active scene.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="46" customHeight="1">
@@ -4677,13 +4677,13 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L12" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Measured: -14.08 LUFS integrated; -1.87 dBTP 4× estimate; -1.87 dBFS sample peak</x:v>
       </x:c>
       <x:c r="M12" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
       </x:c>
       <x:c r="N12" s="21" t="str">
-        <x:v>Keep; verify audible content and loudness in the active scene.</x:v>
+        <x:v>Keep; loudness is hash-bound. Verify audible content, dialogue masking, and lifecycle in the active scene.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="46" customHeight="1">
@@ -4721,13 +4721,13 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L13" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Measured: -9.62 LUFS integrated; 0.03 dBTP 4× estimate; 0 dBFS sample peak</x:v>
       </x:c>
       <x:c r="M13" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
       </x:c>
       <x:c r="N13" s="21" t="str">
-        <x:v>Keep; verify audible content and loudness in the active scene.</x:v>
+        <x:v>Keep; loudness is hash-bound. Verify audible content, dialogue masking, and lifecycle in the active scene.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="46" customHeight="1">
@@ -4765,13 +4765,13 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L14" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Measured: -13.7 LUFS integrated; -0.8 dBTP 4× estimate; -0.8 dBFS sample peak</x:v>
       </x:c>
       <x:c r="M14" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
       </x:c>
       <x:c r="N14" s="21" t="str">
-        <x:v>Keep; verify audible content and loudness in the active scene.</x:v>
+        <x:v>Keep; loudness is hash-bound. Verify audible content, dialogue masking, and lifecycle in the active scene.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="46" customHeight="1">
@@ -4809,13 +4809,13 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L15" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Measured: -13.04 LUFS integrated; -0.97 dBTP 4× estimate; -1.01 dBFS sample peak</x:v>
       </x:c>
       <x:c r="M15" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
       </x:c>
       <x:c r="N15" s="21" t="str">
-        <x:v>Keep; verify audible content and loudness in the active scene.</x:v>
+        <x:v>Keep; loudness is hash-bound. Verify audible content, dialogue masking, and lifecycle in the active scene.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="46" customHeight="1">
@@ -4853,13 +4853,13 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L16" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Measured: -11.43 LUFS integrated; 0.65 dBTP 4× estimate; 0.59 dBFS sample peak</x:v>
       </x:c>
       <x:c r="M16" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
       </x:c>
       <x:c r="N16" s="21" t="str">
-        <x:v>Keep; verify audible content and loudness in the active scene.</x:v>
+        <x:v>Keep; loudness is hash-bound. Verify audible content, dialogue masking, and lifecycle in the active scene.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="46" customHeight="1">
@@ -4897,13 +4897,13 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L17" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Measured: -15.31 LUFS integrated; -3.69 dBTP 4× estimate; -3.69 dBFS sample peak</x:v>
       </x:c>
       <x:c r="M17" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
       </x:c>
       <x:c r="N17" s="21" t="str">
-        <x:v>Keep; verify audible content and loudness in the active scene.</x:v>
+        <x:v>Keep; loudness is hash-bound. Verify audible content, dialogue masking, and lifecycle in the active scene.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="46" customHeight="1">
@@ -4941,7 +4941,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L18" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M18" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -4985,7 +4985,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L19" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M19" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -5029,7 +5029,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L20" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M20" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -5073,7 +5073,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L21" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M21" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -5117,7 +5117,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L22" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M22" s="21" t="str">
         <x:v>No reachable runtime use found</x:v>
@@ -5161,7 +5161,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L23" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M23" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -5205,7 +5205,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L24" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M24" s="21" t="str">
         <x:v>No reachable runtime use found</x:v>
@@ -5249,7 +5249,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L25" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M25" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -5293,7 +5293,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L26" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M26" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -5337,7 +5337,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L27" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M27" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -5381,7 +5381,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L28" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M28" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -5425,7 +5425,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L29" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M29" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -5469,7 +5469,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L30" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M30" s="21" t="str">
         <x:v>No reachable runtime use found</x:v>
@@ -5513,7 +5513,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L31" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M31" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -5557,7 +5557,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L32" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M32" s="21" t="str">
         <x:v>No reachable runtime use found</x:v>
@@ -5601,7 +5601,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L33" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M33" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -5645,7 +5645,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L34" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M34" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -5689,7 +5689,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L35" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M35" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -5733,7 +5733,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L36" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M36" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -5777,7 +5777,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L37" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M37" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -5821,7 +5821,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L38" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M38" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -5865,7 +5865,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L39" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M39" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -5909,7 +5909,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L40" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M40" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -5953,7 +5953,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L41" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M41" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -5997,7 +5997,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L42" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M42" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -6041,7 +6041,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L43" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M43" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -6085,7 +6085,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L44" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M44" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -6129,7 +6129,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L45" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M45" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -6173,7 +6173,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L46" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M46" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -6217,7 +6217,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L47" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M47" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -6261,7 +6261,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L48" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M48" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -6305,7 +6305,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L49" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M49" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -6349,7 +6349,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L50" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M50" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -6393,7 +6393,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L51" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M51" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -6437,7 +6437,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L52" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M52" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -6481,7 +6481,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L53" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M53" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -6525,7 +6525,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L54" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M54" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -6569,7 +6569,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L55" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M55" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -6613,7 +6613,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L56" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M56" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -6657,7 +6657,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L57" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M57" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -6701,7 +6701,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L58" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M58" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -6745,7 +6745,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L59" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M59" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -6789,7 +6789,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L60" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M60" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -6833,7 +6833,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L61" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M61" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -6877,7 +6877,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L62" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M62" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -6921,7 +6921,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L63" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M63" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -6965,7 +6965,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L64" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M64" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -7009,7 +7009,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L65" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M65" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -7053,7 +7053,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L66" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M66" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -7097,7 +7097,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L67" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M67" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -7141,7 +7141,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L68" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M68" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -7185,7 +7185,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L69" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M69" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -7229,7 +7229,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L70" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M70" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -7273,7 +7273,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L71" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M71" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -7317,7 +7317,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L72" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M72" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -7361,7 +7361,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L73" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M73" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -7405,7 +7405,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L74" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M74" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -7449,7 +7449,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L75" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M75" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -7493,7 +7493,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L76" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M76" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -7537,7 +7537,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L77" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M77" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -7581,7 +7581,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L78" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M78" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -7625,7 +7625,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L79" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M79" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -7669,7 +7669,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L80" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M80" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -7713,7 +7713,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L81" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M81" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -7757,7 +7757,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L82" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M82" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -7801,7 +7801,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L83" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M83" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -7845,7 +7845,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L84" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M84" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -7889,7 +7889,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L85" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M85" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -7933,7 +7933,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L86" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M86" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -7977,7 +7977,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L87" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M87" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -8021,7 +8021,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L88" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M88" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -8065,7 +8065,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L89" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M89" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -8109,7 +8109,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L90" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M90" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -8153,7 +8153,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L91" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M91" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -8197,7 +8197,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L92" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M92" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -8241,7 +8241,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L93" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M93" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -8285,7 +8285,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L94" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M94" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -8329,7 +8329,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L95" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M95" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -8373,7 +8373,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L96" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M96" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -8417,7 +8417,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L97" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M97" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -8461,7 +8461,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L98" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M98" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -8505,7 +8505,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L99" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M99" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -8549,7 +8549,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L100" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M100" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -8593,7 +8593,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L101" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M101" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -8637,7 +8637,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L102" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M102" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -8681,7 +8681,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L103" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M103" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -8725,7 +8725,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L104" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M104" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -8769,7 +8769,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L105" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M105" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -8813,7 +8813,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L106" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M106" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -8857,7 +8857,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L107" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M107" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -8901,7 +8901,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L108" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M108" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -8945,7 +8945,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L109" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M109" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -8989,7 +8989,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L110" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M110" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -9033,7 +9033,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L111" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M111" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -9077,7 +9077,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L112" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M112" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -9121,7 +9121,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L113" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M113" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -9165,7 +9165,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L114" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M114" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -9209,7 +9209,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L115" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M115" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -9253,7 +9253,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L116" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M116" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -9297,7 +9297,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L117" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M117" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -9341,7 +9341,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L118" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M118" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -9385,7 +9385,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L119" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M119" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -9429,7 +9429,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L120" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M120" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -9473,7 +9473,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L121" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M121" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -9517,7 +9517,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L122" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M122" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -9561,7 +9561,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L123" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M123" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -9605,7 +9605,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L124" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M124" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -9649,7 +9649,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L125" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M125" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -9693,7 +9693,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L126" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M126" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -9737,7 +9737,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L127" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M127" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -9781,7 +9781,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L128" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M128" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -9825,7 +9825,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L129" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M129" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -9869,7 +9869,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L130" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M130" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -9913,7 +9913,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L131" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M131" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -9957,7 +9957,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L132" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M132" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -10001,7 +10001,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L133" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M133" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -10045,7 +10045,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L134" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M134" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -10089,7 +10089,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L135" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M135" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -10133,7 +10133,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L136" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M136" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -10177,7 +10177,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L137" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M137" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -10221,7 +10221,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L138" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M138" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -10265,7 +10265,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L139" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M139" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -10309,7 +10309,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L140" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M140" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -10353,7 +10353,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L141" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M141" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -10397,7 +10397,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L142" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M142" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -10441,7 +10441,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L143" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M143" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -10485,7 +10485,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L144" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M144" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -10529,7 +10529,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L145" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M145" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -10573,7 +10573,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L146" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M146" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -10617,7 +10617,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L147" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M147" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -10661,7 +10661,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L148" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M148" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -10705,7 +10705,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L149" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M149" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -10749,7 +10749,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L150" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M150" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -10793,7 +10793,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L151" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M151" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -10837,7 +10837,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L152" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M152" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -10881,7 +10881,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L153" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M153" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -10925,7 +10925,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L154" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M154" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -10969,7 +10969,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L155" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M155" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -11013,7 +11013,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L156" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M156" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -11057,7 +11057,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L157" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M157" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -11101,7 +11101,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L158" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M158" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -11145,7 +11145,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L159" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M159" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -11189,7 +11189,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L160" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M160" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -11233,7 +11233,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L161" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M161" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -11277,7 +11277,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L162" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M162" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -11321,7 +11321,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L163" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M163" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -11365,7 +11365,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L164" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M164" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -11409,7 +11409,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L165" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M165" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -11453,7 +11453,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L166" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M166" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -11497,7 +11497,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L167" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M167" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -11541,7 +11541,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L168" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M168" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -11585,7 +11585,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L169" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M169" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -11629,7 +11629,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L170" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M170" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -11673,7 +11673,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L171" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M171" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -11717,7 +11717,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L172" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M172" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -11761,7 +11761,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L173" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M173" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -11805,7 +11805,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L174" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M174" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -11849,7 +11849,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L175" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M175" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -11893,7 +11893,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L176" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M176" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -11937,7 +11937,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L177" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M177" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -11981,7 +11981,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L178" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M178" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -12025,7 +12025,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L179" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M179" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -12069,7 +12069,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L180" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M180" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -12113,7 +12113,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L181" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M181" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -12157,7 +12157,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L182" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M182" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -12201,7 +12201,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L183" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M183" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -12245,7 +12245,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L184" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M184" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -12289,7 +12289,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L185" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M185" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -12333,7 +12333,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L186" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M186" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -12377,7 +12377,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L187" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M187" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -12421,7 +12421,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L188" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M188" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -12465,7 +12465,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L189" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M189" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -12509,7 +12509,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L190" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M190" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -12553,7 +12553,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L191" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M191" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -12597,7 +12597,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L192" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M192" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -12641,7 +12641,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L193" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M193" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -12685,7 +12685,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L194" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M194" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -12729,7 +12729,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L195" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M195" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -12773,7 +12773,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L196" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M196" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -12817,7 +12817,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L197" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M197" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -12861,7 +12861,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L198" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M198" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -12905,7 +12905,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L199" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M199" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -12949,7 +12949,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L200" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M200" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -12993,7 +12993,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L201" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M201" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -13037,7 +13037,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L202" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M202" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -13081,7 +13081,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L203" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M203" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -13125,7 +13125,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L204" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M204" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -13169,7 +13169,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L205" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M205" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -13213,7 +13213,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L206" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M206" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -13257,7 +13257,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L207" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M207" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -13301,7 +13301,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L208" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M208" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -13345,7 +13345,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L209" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M209" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -13389,7 +13389,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L210" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M210" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -13433,7 +13433,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L211" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M211" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -13477,7 +13477,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L212" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M212" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -13521,7 +13521,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L213" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M213" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -13565,7 +13565,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L214" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M214" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -13609,7 +13609,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L215" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M215" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -13653,7 +13653,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L216" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M216" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -13697,7 +13697,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L217" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M217" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -13741,7 +13741,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L218" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M218" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -13785,7 +13785,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L219" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M219" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -13829,7 +13829,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L220" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M220" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -13873,7 +13873,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L221" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M221" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -13917,7 +13917,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L222" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M222" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -13961,7 +13961,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L223" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M223" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -14005,7 +14005,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L224" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M224" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -14049,7 +14049,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L225" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M225" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -14093,7 +14093,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L226" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M226" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -14137,7 +14137,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L227" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M227" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -14181,7 +14181,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L228" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M228" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -14225,7 +14225,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L229" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M229" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -14269,7 +14269,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L230" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M230" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -14313,7 +14313,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L231" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M231" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -14357,7 +14357,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L232" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M232" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -14401,7 +14401,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L233" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M233" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -14445,7 +14445,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L234" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M234" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -14489,7 +14489,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L235" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M235" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -14533,7 +14533,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L236" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M236" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -14577,7 +14577,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L237" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M237" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -14621,7 +14621,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L238" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M238" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -14665,7 +14665,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L239" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M239" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -14709,7 +14709,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L240" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M240" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -14753,7 +14753,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L241" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M241" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -14797,7 +14797,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L242" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M242" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -14841,7 +14841,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L243" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M243" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -14885,7 +14885,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L244" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M244" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -14929,7 +14929,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L245" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M245" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -14973,7 +14973,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L246" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M246" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -15017,7 +15017,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L247" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M247" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -15061,7 +15061,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L248" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M248" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -15105,7 +15105,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L249" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M249" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -15149,7 +15149,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L250" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M250" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -15193,7 +15193,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L251" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M251" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -15237,7 +15237,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L252" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M252" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -15281,7 +15281,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L253" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M253" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -15325,7 +15325,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L254" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M254" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -15369,7 +15369,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L255" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M255" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -15413,7 +15413,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L256" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M256" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -15457,7 +15457,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L257" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M257" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -15501,7 +15501,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L258" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M258" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -15545,7 +15545,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L259" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M259" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -15589,7 +15589,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L260" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M260" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -15633,7 +15633,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L261" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M261" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -15677,7 +15677,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L262" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M262" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -15721,7 +15721,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L263" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M263" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -15765,7 +15765,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L264" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M264" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -15809,7 +15809,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L265" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M265" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -15853,7 +15853,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L266" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M266" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -15897,7 +15897,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L267" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M267" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -15941,7 +15941,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L268" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M268" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -15985,7 +15985,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L269" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M269" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -16029,7 +16029,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L270" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M270" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -16073,7 +16073,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L271" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M271" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -16117,7 +16117,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L272" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M272" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -16161,7 +16161,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L273" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M273" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -16205,7 +16205,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L274" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M274" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -16249,7 +16249,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L275" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M275" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -16293,7 +16293,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L276" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M276" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -16337,7 +16337,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L277" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M277" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -16381,7 +16381,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L278" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M278" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -16425,7 +16425,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L279" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M279" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -16469,7 +16469,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L280" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M280" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -16513,7 +16513,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L281" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M281" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -16557,7 +16557,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L282" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M282" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -16601,7 +16601,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L283" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M283" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -16645,7 +16645,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L284" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M284" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -16689,7 +16689,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L285" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M285" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -16733,7 +16733,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L286" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M286" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -16777,7 +16777,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L287" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M287" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -16821,7 +16821,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L288" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M288" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -16865,7 +16865,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L289" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M289" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -16909,7 +16909,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L290" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M290" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -16953,7 +16953,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L291" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M291" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -16997,7 +16997,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L292" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M292" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -17041,7 +17041,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L293" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M293" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -17085,7 +17085,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L294" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M294" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -17129,7 +17129,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L295" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M295" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -17173,7 +17173,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L296" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M296" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -17217,7 +17217,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L297" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M297" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -17261,7 +17261,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L298" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M298" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -17305,7 +17305,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L299" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M299" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -17349,7 +17349,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L300" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M300" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -17393,7 +17393,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L301" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M301" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -17437,7 +17437,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L302" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M302" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -17481,7 +17481,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L303" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M303" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -17525,7 +17525,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L304" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M304" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -17569,7 +17569,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L305" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M305" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -17613,7 +17613,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L306" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M306" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -17657,7 +17657,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L307" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M307" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -17701,7 +17701,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L308" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M308" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -17745,7 +17745,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L309" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M309" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -17789,7 +17789,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L310" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M310" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -17833,7 +17833,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L311" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Measured: -15.99 LUFS integrated; -1.54 dBTP 4× estimate; -1.58 dBFS sample peak</x:v>
       </x:c>
       <x:c r="M311" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -17877,7 +17877,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L312" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Measured: -12.72 LUFS integrated; 0.14 dBTP 4× estimate; 0 dBFS sample peak</x:v>
       </x:c>
       <x:c r="M312" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -17921,7 +17921,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L313" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Measured: -14.05 LUFS integrated; -0.06 dBTP 4× estimate; -0.08 dBFS sample peak</x:v>
       </x:c>
       <x:c r="M313" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -17965,7 +17965,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L314" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Measured: -16.37 LUFS integrated; -4.17 dBTP 4× estimate; -4.17 dBFS sample peak</x:v>
       </x:c>
       <x:c r="M314" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -18009,7 +18009,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L315" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Measured: -12.21 LUFS integrated; 0.06 dBTP 4× estimate; 0 dBFS sample peak</x:v>
       </x:c>
       <x:c r="M315" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -18053,7 +18053,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L316" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Measured: -11.23 LUFS integrated; -0.23 dBTP 4× estimate; -0.23 dBFS sample peak</x:v>
       </x:c>
       <x:c r="M316" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -18097,7 +18097,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L317" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Measured: -10.04 LUFS integrated; 0.54 dBTP 4× estimate; 0.53 dBFS sample peak</x:v>
       </x:c>
       <x:c r="M317" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -18141,7 +18141,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L318" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Measured: -13.15 LUFS integrated; 0.14 dBTP 4× estimate; 0.13 dBFS sample peak</x:v>
       </x:c>
       <x:c r="M318" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -18185,7 +18185,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L319" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Measured: -14.68 LUFS integrated; -1.86 dBTP 4× estimate; -1.91 dBFS sample peak</x:v>
       </x:c>
       <x:c r="M319" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -18229,7 +18229,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L320" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Measured: -11.22 LUFS integrated; 0 dBTP 4× estimate; 0 dBFS sample peak</x:v>
       </x:c>
       <x:c r="M320" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -18273,7 +18273,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L321" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Measured: -13.46 LUFS integrated; -2.38 dBTP 4× estimate; -2.38 dBFS sample peak</x:v>
       </x:c>
       <x:c r="M321" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -18317,7 +18317,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L322" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Measured: -15.73 LUFS integrated; -3.74 dBTP 4× estimate; -3.74 dBFS sample peak</x:v>
       </x:c>
       <x:c r="M322" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -18361,7 +18361,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L323" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M323" s="21" t="str">
         <x:v>No reachable runtime use found</x:v>
@@ -18405,7 +18405,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L324" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M324" s="21" t="str">
         <x:v>No reachable runtime use found</x:v>
@@ -18449,7 +18449,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L325" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M325" s="21" t="str">
         <x:v>No reachable runtime use found</x:v>
@@ -18493,7 +18493,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L326" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M326" s="21" t="str">
         <x:v>No reachable runtime use found</x:v>
@@ -18537,7 +18537,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L327" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M327" s="21" t="str">
         <x:v>No reachable runtime use found</x:v>
@@ -18581,7 +18581,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L328" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M328" s="21" t="str">
         <x:v>No reachable runtime use found</x:v>
@@ -18625,7 +18625,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L329" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M329" s="21" t="str">
         <x:v>No reachable runtime use found</x:v>
@@ -18669,7 +18669,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L330" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M330" s="21" t="str">
         <x:v>No reachable runtime use found</x:v>
@@ -18713,7 +18713,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L331" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M331" s="21" t="str">
         <x:v>No reachable runtime use found</x:v>
@@ -18757,7 +18757,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L332" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M332" s="21" t="str">
         <x:v>No reachable runtime use found</x:v>
@@ -18801,7 +18801,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L333" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M333" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -18845,7 +18845,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L334" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M334" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -18889,7 +18889,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L335" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M335" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -18933,7 +18933,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L336" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M336" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -18977,7 +18977,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L337" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M337" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -19021,7 +19021,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L338" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M338" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -19065,7 +19065,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L339" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M339" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -19109,7 +19109,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L340" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M340" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -19153,7 +19153,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L341" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M341" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -19197,7 +19197,7 @@
         <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
       </x:c>
       <x:c r="L342" s="21" t="str">
-        <x:v>UNMEASURED — no integrated-LUFS evidence</x:v>
+        <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M342" s="21" t="str">
         <x:v>No source-level issue; active-play receipt pending</x:v>
@@ -19214,7 +19214,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ff686afa0614424"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b307329418845a1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19480,16 +19480,16 @@
         <x:v>Mix / loudness</x:v>
       </x:c>
       <x:c r="D11" s="24" t="str">
-        <x:v>Configured gains are documented, but no integrated-LUFS or true-peak audit exists for radio, venue, driving, and mission masters.</x:v>
+        <x:v>24/24 long-form masters now have hash-bound integrated-LUFS, sample-peak, and 4× intersample peak evidence; configured gains still need active-scene mix review.</x:v>
       </x:c>
       <x:c r="E11" s="24" t="str">
-        <x:v>Cue Inventory duration is measured from files; loudness remains explicitly UNMEASURED.</x:v>
+        <x:v>docs/audits/radio/loudness-measurements.json plus the generated Cue Inventory; the meter makes no production gain changes.</x:v>
       </x:c>
       <x:c r="F11" s="24" t="str">
         <x:v>Tracks at the same configured gain can have very different perceived loudness and mask dialogue.</x:v>
       </x:c>
       <x:c r="G11" s="24" t="str">
-        <x:v>Mechanical: add repeatable loudness analysis; OWNER approves any gain or asset normalization changes.</x:v>
+        <x:v>Mechanical measurement is complete. Add active-play dialogue/overlap receipts; OWNER approves any gain or asset normalization changes.</x:v>
       </x:c>
       <x:c r="H11" s="24" t="str">
         <x:v>Mechanical</x:v>
@@ -19498,7 +19498,7 @@
         <x:v>OWNER for audible mix changes after measurements.</x:v>
       </x:c>
       <x:c r="J11" s="24" t="str">
-        <x:v>OPEN</x:v>
+        <x:v>MEASURED — ACTIVE MIX REVIEW OPEN</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="54" customHeight="1">
@@ -19733,7 +19733,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R29373efccd984022"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcbd978e9baec47d0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19920,10 +19920,10 @@
         <x:v>Add repeatable duration, integrated-loudness, true-peak, and identity evidence</x:v>
       </x:c>
       <x:c r="C10" s="21" t="str">
-        <x:v>tools/radio-audit.mjs; audio QA tooling; generated Cue Inventory</x:v>
+        <x:v>tools/audio-loudness-audit.mjs; docs/audits/radio/loudness-measurements.json; tools/radio-audit.mjs; generated Cue Inventory</x:v>
       </x:c>
       <x:c r="D10" s="21" t="str">
-        <x:v>Approved local analysis/transcription tooling</x:v>
+        <x:v>Existing Playwright Chromium decoder; supervised listening/transcription for content identity</x:v>
       </x:c>
       <x:c r="E10" s="21" t="str">
         <x:v>Medium</x:v>
@@ -19932,7 +19932,7 @@
         <x:v>Every retained master has measured duration/LUFS/peak and verified content or an explicit exception</x:v>
       </x:c>
       <x:c r="G10" s="21" t="str">
-        <x:v>PARTIAL — duration only</x:v>
+        <x:v>LOUDNESS DONE — CONTENT IDENTITY PENDING</x:v>
       </x:c>
       <x:c r="H10" s="21" t="str"/>
     </x:row>
@@ -20040,7 +20040,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f47a172fa604a4f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ad5707d6a9f4ad8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat(radio): verify content and close receiver gaps
Owner handoff: audit every campaign radio, venue score, vehicle cue, stinger, and silence without silently replacing owner-selected music.

Updated the generated 31-beat workbook/CSVs for the persistent Luxury and Mansion receivers, corrected stale one-station documentation, and added hash-bound Scribe evidence for all 298 spoken radio/news assets. Three unclear announcer takes were replaced in the preceding audio commit and now match; all remaining number/filler/pronunciation variants normalize deterministically. The audit now distinguishes 298/298 verified speech from 24/24 loudness-measured but owner-reviewed music masters, retains four legacy identity orphans as explicit OWNER decisions, and records zero missing assets. Verified 26/26 focused contracts, audit/check generators, loudness hashes, 298/298 content receipts, five rendered workbook sheets, and zero formula errors.
</commit_message>
<xml_diff>
--- a/docs/audits/SQUATCHSMASH-RADIO-AUDIT.xlsx
+++ b/docs/audits/SQUATCHSMASH-RADIO-AUDIT.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scene Timeline" sheetId="1" r:id="Re97fc961620f4b0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Station Catalog" sheetId="2" r:id="R13e72fa051ce4744"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cue Inventory" sheetId="3" r:id="R7ff68e4b5cb54587"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Problems and Decisions" sheetId="4" r:id="R652078f99ae04668"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revamp Plan" sheetId="5" r:id="Rc93aad9db3204e1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scene Timeline" sheetId="1" r:id="R36b1b4ba8b8e4009"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Station Catalog" sheetId="2" r:id="R5b92ed2b17a746bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cue Inventory" sheetId="3" r:id="R0d5cf8d5b2924182"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Problems and Decisions" sheetId="4" r:id="R8887422464b24d46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revamp Plan" sheetId="5" r:id="Rbf6b0c7f8d9d450a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -585,7 +585,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="10" t="str">
-        <x:v>43 data rows · Generated by tools/radio-audit.mjs · Source-only findings remain explicitly marked for active-play/loudness/content verification.</x:v>
+        <x:v>43 data rows · Generated by tools/radio-audit.mjs · Active-play mix, music identity, provenance, and owner decisions remain explicitly marked.</x:v>
       </x:c>
       <x:c r="B3" s="10"/>
       <x:c r="C3" s="10"/>
@@ -2406,7 +2406,7 @@
         <x:v>Luxury apartment</x:v>
       </x:c>
       <x:c r="H28" s="21" t="str">
-        <x:v>Physical 97.8 receiver · scene-local state</x:v>
+        <x:v>Physical 97.8 receiver · luxury_apartment</x:v>
       </x:c>
       <x:c r="I28" s="21" t="str">
         <x:v>97.8 THE SQUATCH</x:v>
@@ -2442,22 +2442,22 @@
         <x:v>Diegetic receiver</x:v>
       </x:c>
       <x:c r="T28" s="21" t="str">
-        <x:v>MEDIUM — state resets on reload</x:v>
+        <x:v>LOW/MEDIUM — verify against scene music</x:v>
       </x:c>
       <x:c r="U28" s="21" t="str">
         <x:v>WIRED · LIVE RECEIVER</x:v>
       </x:c>
       <x:c r="V28" s="21" t="str">
-        <x:v>Eligible: good-ole-days.mp3, through-the-night.mp3, 10-drunk-cigarettes.mp3, i-aint-gay.mp3, nehoo-with-a-guu.mp3; not campaign-persisted.</x:v>
+        <x:v>Eligible: good-ole-days.mp3, through-the-night.mp3, 10-drunk-cigarettes.mp3, i-aint-gay.mp3, nehoo-with-a-guu.mp3; campaign-persisted.</x:v>
       </x:c>
       <x:c r="W28" s="21" t="str">
-        <x:v>Mechanical: give this receiver the shared campaign adapter if reload continuity is intended.</x:v>
+        <x:v>Keep; add active-play overlap receipt.</x:v>
       </x:c>
       <x:c r="X28" s="21" t="str">
         <x:v>No for receiver mechanics; OWNER only for playlist identity.</x:v>
       </x:c>
       <x:c r="Y28" s="21" t="str">
-        <x:v>Live; persistence gap open</x:v>
+        <x:v>Live; active-play audit pending</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="54" customHeight="1">
@@ -2714,7 +2714,7 @@
         <x:v>Luxury apartment</x:v>
       </x:c>
       <x:c r="H32" s="21" t="str">
-        <x:v>Physical 97.8 receiver · scene-local state</x:v>
+        <x:v>Physical 97.8 receiver · luxury_apartment</x:v>
       </x:c>
       <x:c r="I32" s="21" t="str">
         <x:v>97.8 THE SQUATCH</x:v>
@@ -2750,22 +2750,22 @@
         <x:v>Diegetic receiver</x:v>
       </x:c>
       <x:c r="T32" s="21" t="str">
-        <x:v>MEDIUM — state resets on reload</x:v>
+        <x:v>LOW/MEDIUM — verify against scene music</x:v>
       </x:c>
       <x:c r="U32" s="21" t="str">
         <x:v>WIRED · LIVE RECEIVER</x:v>
       </x:c>
       <x:c r="V32" s="21" t="str">
-        <x:v>Eligible: good-ole-days.mp3, through-the-night.mp3, 10-drunk-cigarettes.mp3, i-aint-gay.mp3, nehoo-with-a-guu.mp3; not campaign-persisted.</x:v>
+        <x:v>Eligible: good-ole-days.mp3, through-the-night.mp3, 10-drunk-cigarettes.mp3, i-aint-gay.mp3, nehoo-with-a-guu.mp3; campaign-persisted.</x:v>
       </x:c>
       <x:c r="W32" s="21" t="str">
-        <x:v>Mechanical: give this receiver the shared campaign adapter if reload continuity is intended.</x:v>
+        <x:v>Keep; add active-play overlap receipt.</x:v>
       </x:c>
       <x:c r="X32" s="21" t="str">
         <x:v>No for receiver mechanics; OWNER only for playlist identity.</x:v>
       </x:c>
       <x:c r="Y32" s="21" t="str">
-        <x:v>Live; persistence gap open</x:v>
+        <x:v>Live; active-play audit pending</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="54" customHeight="1">
@@ -2791,7 +2791,7 @@
         <x:v>Luxury apartment</x:v>
       </x:c>
       <x:c r="H33" s="21" t="str">
-        <x:v>Physical 97.8 receiver · scene-local state</x:v>
+        <x:v>Physical 97.8 receiver · luxury_apartment</x:v>
       </x:c>
       <x:c r="I33" s="21" t="str">
         <x:v>97.8 THE SQUATCH</x:v>
@@ -2827,22 +2827,22 @@
         <x:v>Diegetic receiver</x:v>
       </x:c>
       <x:c r="T33" s="21" t="str">
-        <x:v>MEDIUM — state resets on reload</x:v>
+        <x:v>LOW/MEDIUM — verify against scene music</x:v>
       </x:c>
       <x:c r="U33" s="21" t="str">
         <x:v>WIRED · LIVE RECEIVER</x:v>
       </x:c>
       <x:c r="V33" s="21" t="str">
-        <x:v>Eligible: good-ole-days.mp3, through-the-night.mp3, 10-drunk-cigarettes.mp3, i-aint-gay.mp3, nehoo-with-a-guu.mp3; not campaign-persisted.</x:v>
+        <x:v>Eligible: good-ole-days.mp3, through-the-night.mp3, 10-drunk-cigarettes.mp3, i-aint-gay.mp3, nehoo-with-a-guu.mp3; campaign-persisted.</x:v>
       </x:c>
       <x:c r="W33" s="21" t="str">
-        <x:v>Mechanical: give this receiver the shared campaign adapter if reload continuity is intended.</x:v>
+        <x:v>Keep; add active-play overlap receipt.</x:v>
       </x:c>
       <x:c r="X33" s="21" t="str">
         <x:v>No for receiver mechanics; OWNER only for playlist identity.</x:v>
       </x:c>
       <x:c r="Y33" s="21" t="str">
-        <x:v>Live; persistence gap open</x:v>
+        <x:v>Live; active-play audit pending</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="54" customHeight="1">
@@ -2945,7 +2945,7 @@
         <x:v>Luxury apartment</x:v>
       </x:c>
       <x:c r="H35" s="21" t="str">
-        <x:v>Physical 97.8 receiver · scene-local state</x:v>
+        <x:v>Physical 97.8 receiver · luxury_apartment</x:v>
       </x:c>
       <x:c r="I35" s="21" t="str">
         <x:v>97.8 THE SQUATCH</x:v>
@@ -2981,22 +2981,22 @@
         <x:v>Diegetic receiver</x:v>
       </x:c>
       <x:c r="T35" s="21" t="str">
-        <x:v>MEDIUM — state resets on reload</x:v>
+        <x:v>LOW/MEDIUM — verify against scene music</x:v>
       </x:c>
       <x:c r="U35" s="21" t="str">
         <x:v>WIRED · LIVE RECEIVER</x:v>
       </x:c>
       <x:c r="V35" s="21" t="str">
-        <x:v>Eligible: good-ole-days.mp3, through-the-night.mp3, 10-drunk-cigarettes.mp3, i-aint-gay.mp3, nehoo-with-a-guu.mp3; not campaign-persisted.</x:v>
+        <x:v>Eligible: good-ole-days.mp3, through-the-night.mp3, 10-drunk-cigarettes.mp3, i-aint-gay.mp3, nehoo-with-a-guu.mp3; campaign-persisted.</x:v>
       </x:c>
       <x:c r="W35" s="21" t="str">
-        <x:v>Mechanical: give this receiver the shared campaign adapter if reload continuity is intended.</x:v>
+        <x:v>Keep; add active-play overlap receipt.</x:v>
       </x:c>
       <x:c r="X35" s="21" t="str">
         <x:v>No for receiver mechanics; OWNER only for playlist identity.</x:v>
       </x:c>
       <x:c r="Y35" s="21" t="str">
-        <x:v>Live; persistence gap open</x:v>
+        <x:v>Live; active-play audit pending</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="54" customHeight="1">
@@ -3099,7 +3099,7 @@
         <x:v>Lou’s mansion and Silent Squatch cellar</x:v>
       </x:c>
       <x:c r="H37" s="21" t="str">
-        <x:v>Physical 97.8 receiver · scene-local state</x:v>
+        <x:v>Physical 97.8 receiver · mansion_house</x:v>
       </x:c>
       <x:c r="I37" s="21" t="str">
         <x:v>97.8 THE SQUATCH</x:v>
@@ -3135,22 +3135,22 @@
         <x:v>Diegetic receiver</x:v>
       </x:c>
       <x:c r="T37" s="21" t="str">
-        <x:v>MEDIUM — state resets on reload</x:v>
+        <x:v>LOW/MEDIUM — verify against scene music</x:v>
       </x:c>
       <x:c r="U37" s="21" t="str">
         <x:v>WIRED · LIVE RECEIVER</x:v>
       </x:c>
       <x:c r="V37" s="21" t="str">
-        <x:v>Eligible: good-ole-days.mp3, through-the-night.mp3, daydream-diner-2.mp3, 10-drunk-cigarettes.mp3, i-aint-gay.mp3, nehoo-with-a-guu.mp3; not campaign-persisted.</x:v>
+        <x:v>Eligible: good-ole-days.mp3, through-the-night.mp3, daydream-diner-2.mp3, 10-drunk-cigarettes.mp3, i-aint-gay.mp3, nehoo-with-a-guu.mp3; campaign-persisted.</x:v>
       </x:c>
       <x:c r="W37" s="21" t="str">
-        <x:v>Mechanical: give this receiver the shared campaign adapter if reload continuity is intended.</x:v>
+        <x:v>Keep; add active-play overlap receipt.</x:v>
       </x:c>
       <x:c r="X37" s="21" t="str">
         <x:v>No for receiver mechanics; OWNER only for playlist identity.</x:v>
       </x:c>
       <x:c r="Y37" s="21" t="str">
-        <x:v>Live; persistence gap open</x:v>
+        <x:v>Live; active-play audit pending</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="54" customHeight="1">
@@ -3176,7 +3176,7 @@
         <x:v>Lou’s mansion and Silent Squatch cellar</x:v>
       </x:c>
       <x:c r="H38" s="21" t="str">
-        <x:v>Physical 97.8 receiver · scene-local state</x:v>
+        <x:v>Physical 97.8 receiver · mansion_house</x:v>
       </x:c>
       <x:c r="I38" s="21" t="str">
         <x:v>97.8 THE SQUATCH</x:v>
@@ -3212,22 +3212,22 @@
         <x:v>Diegetic receiver</x:v>
       </x:c>
       <x:c r="T38" s="21" t="str">
-        <x:v>MEDIUM — state resets on reload</x:v>
+        <x:v>LOW/MEDIUM — verify against scene music</x:v>
       </x:c>
       <x:c r="U38" s="21" t="str">
         <x:v>WIRED · LIVE RECEIVER</x:v>
       </x:c>
       <x:c r="V38" s="21" t="str">
-        <x:v>Eligible: good-ole-days.mp3, through-the-night.mp3, daydream-diner-2.mp3, 10-drunk-cigarettes.mp3, i-aint-gay.mp3, nehoo-with-a-guu.mp3; not campaign-persisted.</x:v>
+        <x:v>Eligible: good-ole-days.mp3, through-the-night.mp3, daydream-diner-2.mp3, 10-drunk-cigarettes.mp3, i-aint-gay.mp3, nehoo-with-a-guu.mp3; campaign-persisted.</x:v>
       </x:c>
       <x:c r="W38" s="21" t="str">
-        <x:v>Mechanical: give this receiver the shared campaign adapter if reload continuity is intended.</x:v>
+        <x:v>Keep; add active-play overlap receipt.</x:v>
       </x:c>
       <x:c r="X38" s="21" t="str">
         <x:v>No for receiver mechanics; OWNER only for playlist identity.</x:v>
       </x:c>
       <x:c r="Y38" s="21" t="str">
-        <x:v>Live; persistence gap open</x:v>
+        <x:v>Live; active-play audit pending</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="54" customHeight="1">
@@ -3638,7 +3638,7 @@
         <x:v>Repaired Lou’s mansion</x:v>
       </x:c>
       <x:c r="H44" s="21" t="str">
-        <x:v>Physical 97.8 receiver · scene-local state</x:v>
+        <x:v>Physical 97.8 receiver · mansion_house</x:v>
       </x:c>
       <x:c r="I44" s="21" t="str">
         <x:v>97.8 THE SQUATCH</x:v>
@@ -3674,22 +3674,22 @@
         <x:v>Diegetic receiver</x:v>
       </x:c>
       <x:c r="T44" s="21" t="str">
-        <x:v>MEDIUM — state resets on reload</x:v>
+        <x:v>LOW/MEDIUM — verify against scene music</x:v>
       </x:c>
       <x:c r="U44" s="21" t="str">
         <x:v>WIRED · LIVE RECEIVER</x:v>
       </x:c>
       <x:c r="V44" s="21" t="str">
-        <x:v>Eligible: good-ole-days.mp3, through-the-night.mp3, daydream-diner-2.mp3, 10-drunk-cigarettes.mp3, i-aint-gay.mp3, nehoo-with-a-guu.mp3; not campaign-persisted.</x:v>
+        <x:v>Eligible: good-ole-days.mp3, through-the-night.mp3, daydream-diner-2.mp3, 10-drunk-cigarettes.mp3, i-aint-gay.mp3, nehoo-with-a-guu.mp3; campaign-persisted.</x:v>
       </x:c>
       <x:c r="W44" s="21" t="str">
-        <x:v>Mechanical: give this receiver the shared campaign adapter if reload continuity is intended.</x:v>
+        <x:v>Keep; add active-play overlap receipt.</x:v>
       </x:c>
       <x:c r="X44" s="21" t="str">
         <x:v>No for receiver mechanics; OWNER only for playlist identity.</x:v>
       </x:c>
       <x:c r="Y44" s="21" t="str">
-        <x:v>Live; persistence gap open</x:v>
+        <x:v>Live; active-play audit pending</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="54" customHeight="1">
@@ -3792,7 +3792,7 @@
         <x:v>Luxury apartment</x:v>
       </x:c>
       <x:c r="H46" s="21" t="str">
-        <x:v>Physical 97.8 receiver · scene-local state</x:v>
+        <x:v>Physical 97.8 receiver · luxury_apartment</x:v>
       </x:c>
       <x:c r="I46" s="21" t="str">
         <x:v>97.8 THE SQUATCH</x:v>
@@ -3828,22 +3828,22 @@
         <x:v>Diegetic receiver</x:v>
       </x:c>
       <x:c r="T46" s="21" t="str">
-        <x:v>MEDIUM — state resets on reload</x:v>
+        <x:v>LOW/MEDIUM — verify against scene music</x:v>
       </x:c>
       <x:c r="U46" s="21" t="str">
         <x:v>WIRED · LIVE RECEIVER</x:v>
       </x:c>
       <x:c r="V46" s="21" t="str">
-        <x:v>Eligible: good-ole-days.mp3, through-the-night.mp3, 10-drunk-cigarettes.mp3, i-aint-gay.mp3, nehoo-with-a-guu.mp3; not campaign-persisted.</x:v>
+        <x:v>Eligible: good-ole-days.mp3, through-the-night.mp3, 10-drunk-cigarettes.mp3, i-aint-gay.mp3, nehoo-with-a-guu.mp3; campaign-persisted.</x:v>
       </x:c>
       <x:c r="W46" s="21" t="str">
-        <x:v>Mechanical: give this receiver the shared campaign adapter if reload continuity is intended.</x:v>
+        <x:v>Keep; add active-play overlap receipt.</x:v>
       </x:c>
       <x:c r="X46" s="21" t="str">
         <x:v>No for receiver mechanics; OWNER only for playlist identity.</x:v>
       </x:c>
       <x:c r="Y46" s="21" t="str">
-        <x:v>Live; persistence gap open</x:v>
+        <x:v>Live; active-play audit pending</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="54" customHeight="1">
@@ -4008,7 +4008,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51349b543a82474a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re332e63e7a9e4173"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4068,7 +4068,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="10" t="str">
-        <x:v>3 data rows · Generated by tools/radio-audit.mjs · Source-only findings remain explicitly marked for active-play/loudness/content verification.</x:v>
+        <x:v>3 data rows · Generated by tools/radio-audit.mjs · Active-play mix, music identity, provenance, and owner decisions remain explicitly marked.</x:v>
       </x:c>
       <x:c r="B3" s="10"/>
       <x:c r="C3" s="10"/>
@@ -4255,7 +4255,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77ec43683e3741dd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4758d816acb74388"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4318,7 +4318,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="10" t="str">
-        <x:v>337 data rows · Generated by tools/radio-audit.mjs · Source-only findings remain explicitly marked for active-play/loudness/content verification.</x:v>
+        <x:v>337 data rows · Generated by tools/radio-audit.mjs · Active-play mix, music identity, provenance, and owner decisions remain explicitly marked.</x:v>
       </x:c>
       <x:c r="B3" s="10"/>
       <x:c r="C3" s="10"/>
@@ -4410,7 +4410,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K6" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>OWNER LISTEN — long-form music identity is not inferred from its filename or speech transcription</x:v>
       </x:c>
       <x:c r="L6" s="21" t="str">
         <x:v>Measured: -13.69 LUFS integrated; 0.08 dBTP 4× estimate; 0.08 dBFS sample peak</x:v>
@@ -4454,7 +4454,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K7" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>OWNER LISTEN — long-form music identity is not inferred from its filename or speech transcription</x:v>
       </x:c>
       <x:c r="L7" s="21" t="str">
         <x:v>Measured: -14.07 LUFS integrated; -0.06 dBTP 4× estimate; -0.09 dBFS sample peak</x:v>
@@ -4498,7 +4498,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K8" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>OWNER LISTEN — long-form music identity is not inferred from its filename or speech transcription</x:v>
       </x:c>
       <x:c r="L8" s="21" t="str">
         <x:v>Measured: -16.04 LUFS integrated; -5.79 dBTP 4× estimate; -5.92 dBFS sample peak</x:v>
@@ -4542,7 +4542,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K9" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>OWNER LISTEN — long-form music identity is not inferred from its filename or speech transcription</x:v>
       </x:c>
       <x:c r="L9" s="21" t="str">
         <x:v>Measured: -12.09 LUFS integrated; -0.45 dBTP 4× estimate; -0.45 dBFS sample peak</x:v>
@@ -4586,7 +4586,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K10" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>OWNER LISTEN — long-form music identity is not inferred from its filename or speech transcription</x:v>
       </x:c>
       <x:c r="L10" s="21" t="str">
         <x:v>Measured: -12.2 LUFS integrated; -1.14 dBTP 4× estimate; -1.14 dBFS sample peak</x:v>
@@ -4630,7 +4630,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K11" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>OWNER LISTEN — long-form music identity is not inferred from its filename or speech transcription</x:v>
       </x:c>
       <x:c r="L11" s="21" t="str">
         <x:v>Measured: -12.58 LUFS integrated; -0.95 dBTP 4× estimate; -1.08 dBFS sample peak</x:v>
@@ -4674,7 +4674,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K12" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>OWNER LISTEN — long-form music identity is not inferred from its filename or speech transcription</x:v>
       </x:c>
       <x:c r="L12" s="21" t="str">
         <x:v>Measured: -14.08 LUFS integrated; -1.87 dBTP 4× estimate; -1.87 dBFS sample peak</x:v>
@@ -4718,7 +4718,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K13" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>OWNER LISTEN — long-form music identity is not inferred from its filename or speech transcription</x:v>
       </x:c>
       <x:c r="L13" s="21" t="str">
         <x:v>Measured: -9.62 LUFS integrated; 0.03 dBTP 4× estimate; 0 dBFS sample peak</x:v>
@@ -4762,7 +4762,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K14" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>OWNER LISTEN — long-form music identity is not inferred from its filename or speech transcription</x:v>
       </x:c>
       <x:c r="L14" s="21" t="str">
         <x:v>Measured: -13.7 LUFS integrated; -0.8 dBTP 4× estimate; -0.8 dBFS sample peak</x:v>
@@ -4806,7 +4806,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K15" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>OWNER LISTEN — long-form music identity is not inferred from its filename or speech transcription</x:v>
       </x:c>
       <x:c r="L15" s="21" t="str">
         <x:v>Measured: -13.04 LUFS integrated; -0.97 dBTP 4× estimate; -1.01 dBFS sample peak</x:v>
@@ -4850,7 +4850,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K16" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>OWNER LISTEN — long-form music identity is not inferred from its filename or speech transcription</x:v>
       </x:c>
       <x:c r="L16" s="21" t="str">
         <x:v>Measured: -11.43 LUFS integrated; 0.65 dBTP 4× estimate; 0.59 dBFS sample peak</x:v>
@@ -4894,7 +4894,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K17" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>OWNER LISTEN — long-form music identity is not inferred from its filename or speech transcription</x:v>
       </x:c>
       <x:c r="L17" s="21" t="str">
         <x:v>Measured: -15.31 LUFS integrated; -3.69 dBTP 4× estimate; -3.69 dBFS sample peak</x:v>
@@ -4938,7 +4938,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K18" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>NON-SPEECH — transcription is not applicable; inspect the authored prompt and active playback</x:v>
       </x:c>
       <x:c r="L18" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -4982,7 +4982,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K19" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>NON-SPEECH — transcription is not applicable; inspect the authored prompt and active playback</x:v>
       </x:c>
       <x:c r="L19" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -5026,7 +5026,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K20" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>NON-SPEECH — transcription is not applicable; inspect the authored prompt and active playback</x:v>
       </x:c>
       <x:c r="L20" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -5070,7 +5070,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K21" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>NON-SPEECH — transcription is not applicable; inspect the authored prompt and active playback</x:v>
       </x:c>
       <x:c r="L21" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -5114,7 +5114,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K22" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L22" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -5158,7 +5158,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K23" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L23" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -5202,7 +5202,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K24" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L24" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -5246,7 +5246,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K25" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>NON-SPEECH — transcription is not applicable; inspect the authored prompt and active playback</x:v>
       </x:c>
       <x:c r="L25" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -5290,7 +5290,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K26" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>NON-SPEECH — transcription is not applicable; inspect the authored prompt and active playback</x:v>
       </x:c>
       <x:c r="L26" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -5334,7 +5334,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K27" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>NON-SPEECH — transcription is not applicable; inspect the authored prompt and active playback</x:v>
       </x:c>
       <x:c r="L27" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -5378,7 +5378,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K28" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>NON-SPEECH — transcription is not applicable; inspect the authored prompt and active playback</x:v>
       </x:c>
       <x:c r="L28" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -5422,7 +5422,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K29" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>NON-SPEECH — transcription is not applicable; inspect the authored prompt and active playback</x:v>
       </x:c>
       <x:c r="L29" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -5466,7 +5466,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K30" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>NON-SPEECH — transcription is not applicable; inspect the authored prompt and active playback</x:v>
       </x:c>
       <x:c r="L30" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -5510,7 +5510,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K31" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>NON-SPEECH — transcription is not applicable; inspect the authored prompt and active playback</x:v>
       </x:c>
       <x:c r="L31" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -5554,7 +5554,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K32" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>NON-SPEECH — transcription is not applicable; inspect the authored prompt and active playback</x:v>
       </x:c>
       <x:c r="L32" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -5586,7 +5586,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="G33" s="21" t="n">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="H33" s="21" t="str">
         <x:v>airstrip_smuggling; apartment; bada_bing_one; bada_bing_two; countryside_cabin; luxury_apartment; mansion; mansion_return; no_wake; silver_pines</x:v>
@@ -5598,7 +5598,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K33" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>NON-SPEECH — transcription is not applicable; inspect the authored prompt and active playback</x:v>
       </x:c>
       <x:c r="L33" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -5642,7 +5642,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K34" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>NON-SPEECH — transcription is not applicable; inspect the authored prompt and active playback</x:v>
       </x:c>
       <x:c r="L34" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -5686,7 +5686,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K35" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>NON-SPEECH — transcription is not applicable; inspect the authored prompt and active playback</x:v>
       </x:c>
       <x:c r="L35" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -5730,7 +5730,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K36" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L36" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -5774,7 +5774,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K37" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L37" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -5818,7 +5818,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K38" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L38" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -5862,7 +5862,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K39" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L39" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -5906,7 +5906,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K40" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L40" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -5950,7 +5950,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K41" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L41" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -5994,7 +5994,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K42" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L42" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -6038,7 +6038,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K43" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L43" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -6082,7 +6082,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K44" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L44" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -6105,7 +6105,7 @@
         <x:v>MP3</x:v>
       </x:c>
       <x:c r="D45" s="21" t="n">
-        <x:v>11.494</x:v>
+        <x:v>7.445</x:v>
       </x:c>
       <x:c r="E45" s="21" t="str">
         <x:v>Voice: announcer. License/source field not recorded in manifest.</x:v>
@@ -6126,7 +6126,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K45" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L45" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -6170,7 +6170,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K46" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L46" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -6214,7 +6214,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K47" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L47" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -6258,7 +6258,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K48" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L48" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -6302,7 +6302,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K49" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L49" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -6346,7 +6346,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K50" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L50" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -6390,7 +6390,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K51" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L51" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -6434,7 +6434,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K52" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L52" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -6478,7 +6478,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K53" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L53" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -6522,7 +6522,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K54" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L54" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -6566,7 +6566,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K55" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.9771)</x:v>
       </x:c>
       <x:c r="L55" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -6610,7 +6610,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K56" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L56" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -6654,7 +6654,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K57" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L57" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -6698,7 +6698,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K58" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L58" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -6742,7 +6742,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K59" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L59" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -6786,7 +6786,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K60" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L60" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -6830,7 +6830,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K61" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L61" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -6874,7 +6874,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K62" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.9111)</x:v>
       </x:c>
       <x:c r="L62" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -6918,7 +6918,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K63" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L63" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -6962,7 +6962,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K64" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L64" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -7006,7 +7006,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K65" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L65" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -7050,7 +7050,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K66" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.9577)</x:v>
       </x:c>
       <x:c r="L66" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -7094,7 +7094,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K67" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L67" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -7138,7 +7138,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K68" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.8667)</x:v>
       </x:c>
       <x:c r="L68" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -7182,7 +7182,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K69" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L69" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -7226,7 +7226,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K70" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L70" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -7270,7 +7270,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K71" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L71" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -7314,7 +7314,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K72" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L72" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -7358,7 +7358,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K73" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L73" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -7402,7 +7402,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K74" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L74" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -7446,7 +7446,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K75" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L75" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -7490,7 +7490,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K76" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L76" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -7534,7 +7534,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K77" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L77" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -7578,7 +7578,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K78" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L78" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -7622,7 +7622,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K79" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L79" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -7666,7 +7666,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K80" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L80" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -7710,7 +7710,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K81" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.9919)</x:v>
       </x:c>
       <x:c r="L81" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -7754,7 +7754,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K82" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L82" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -7798,7 +7798,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K83" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L83" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -7842,7 +7842,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K84" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L84" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -7886,7 +7886,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K85" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L85" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -7930,7 +7930,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K86" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.8846)</x:v>
       </x:c>
       <x:c r="L86" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -7974,7 +7974,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K87" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L87" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -8018,7 +8018,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K88" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.9826)</x:v>
       </x:c>
       <x:c r="L88" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -8062,7 +8062,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K89" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L89" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -8106,7 +8106,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K90" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.9852)</x:v>
       </x:c>
       <x:c r="L90" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -8150,7 +8150,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K91" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L91" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -8194,7 +8194,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K92" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.9832)</x:v>
       </x:c>
       <x:c r="L92" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -8238,7 +8238,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K93" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L93" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -8282,7 +8282,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K94" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L94" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -8326,7 +8326,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K95" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.9483)</x:v>
       </x:c>
       <x:c r="L95" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -8370,7 +8370,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K96" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.9783)</x:v>
       </x:c>
       <x:c r="L96" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -8414,7 +8414,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K97" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L97" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -8458,7 +8458,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K98" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L98" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -8502,7 +8502,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K99" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L99" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -8546,7 +8546,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K100" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L100" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -8590,7 +8590,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K101" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L101" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -8634,7 +8634,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K102" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L102" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -8678,7 +8678,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K103" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L103" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -8722,7 +8722,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K104" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L104" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -8766,7 +8766,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K105" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L105" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -8810,7 +8810,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K106" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L106" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -8854,7 +8854,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K107" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L107" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -8898,7 +8898,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K108" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.9897)</x:v>
       </x:c>
       <x:c r="L108" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -8921,7 +8921,7 @@
         <x:v>MP3</x:v>
       </x:c>
       <x:c r="D109" s="21" t="n">
-        <x:v>6.296</x:v>
+        <x:v>4.049</x:v>
       </x:c>
       <x:c r="E109" s="21" t="str">
         <x:v>Voice: announcer. License/source field not recorded in manifest.</x:v>
@@ -8942,7 +8942,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K109" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L109" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -8986,7 +8986,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K110" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L110" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -9030,7 +9030,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K111" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L111" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -9074,7 +9074,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K112" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L112" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -9118,7 +9118,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K113" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L113" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -9162,7 +9162,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K114" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.8846)</x:v>
       </x:c>
       <x:c r="L114" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -9185,7 +9185,7 @@
         <x:v>MP3</x:v>
       </x:c>
       <x:c r="D115" s="21" t="n">
-        <x:v>9.874</x:v>
+        <x:v>9.352</x:v>
       </x:c>
       <x:c r="E115" s="21" t="str">
         <x:v>Voice: announcer. License/source field not recorded in manifest.</x:v>
@@ -9206,7 +9206,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K115" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.9459)</x:v>
       </x:c>
       <x:c r="L115" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -9250,7 +9250,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K116" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L116" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -9294,7 +9294,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K117" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L117" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -9338,7 +9338,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K118" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L118" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -9382,7 +9382,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K119" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L119" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -9426,7 +9426,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K120" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L120" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -9470,7 +9470,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K121" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L121" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -9514,7 +9514,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K122" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L122" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -9558,7 +9558,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K123" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L123" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -9602,7 +9602,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K124" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L124" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -9646,7 +9646,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K125" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L125" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -9690,7 +9690,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K126" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.9835)</x:v>
       </x:c>
       <x:c r="L126" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -9734,7 +9734,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K127" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L127" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -9778,7 +9778,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K128" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L128" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -9822,7 +9822,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K129" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L129" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -9866,7 +9866,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K130" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L130" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -9910,7 +9910,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K131" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L131" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -9954,7 +9954,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K132" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L132" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -9998,7 +9998,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K133" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L133" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -10042,7 +10042,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K134" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.9032)</x:v>
       </x:c>
       <x:c r="L134" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -10086,7 +10086,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K135" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L135" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -10130,7 +10130,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K136" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L136" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -10174,7 +10174,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K137" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L137" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -10218,7 +10218,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K138" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L138" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -10262,7 +10262,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K139" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L139" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -10306,7 +10306,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K140" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.9153)</x:v>
       </x:c>
       <x:c r="L140" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -10350,7 +10350,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K141" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L141" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -10394,7 +10394,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K142" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L142" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -10438,7 +10438,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K143" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.9182)</x:v>
       </x:c>
       <x:c r="L143" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -10482,7 +10482,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K144" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.9859)</x:v>
       </x:c>
       <x:c r="L144" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -10526,7 +10526,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K145" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L145" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -10570,7 +10570,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K146" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L146" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -10614,7 +10614,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K147" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L147" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -10658,7 +10658,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K148" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L148" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -10702,7 +10702,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K149" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.9737)</x:v>
       </x:c>
       <x:c r="L149" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -10746,7 +10746,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K150" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L150" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -10790,7 +10790,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K151" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L151" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -10834,7 +10834,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K152" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L152" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -10878,7 +10878,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K153" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L153" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -10922,7 +10922,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K154" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L154" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -10966,7 +10966,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K155" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L155" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -11010,7 +11010,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K156" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L156" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -11054,7 +11054,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K157" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L157" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -11098,7 +11098,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K158" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L158" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -11142,7 +11142,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K159" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L159" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -11186,7 +11186,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K160" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L160" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -11230,7 +11230,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K161" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L161" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -11274,7 +11274,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K162" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L162" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -11318,7 +11318,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K163" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L163" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -11362,7 +11362,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K164" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.9524)</x:v>
       </x:c>
       <x:c r="L164" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -11406,7 +11406,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K165" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L165" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -11450,7 +11450,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K166" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.9545)</x:v>
       </x:c>
       <x:c r="L166" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -11494,7 +11494,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K167" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L167" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -11538,7 +11538,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K168" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L168" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -11582,7 +11582,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K169" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L169" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -11626,7 +11626,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K170" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L170" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -11670,7 +11670,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K171" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L171" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -11714,7 +11714,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K172" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.8689)</x:v>
       </x:c>
       <x:c r="L172" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -11758,7 +11758,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K173" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L173" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -11802,7 +11802,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K174" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L174" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -11846,7 +11846,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K175" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.8889)</x:v>
       </x:c>
       <x:c r="L175" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -11890,7 +11890,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K176" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L176" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -11934,7 +11934,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K177" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L177" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -11978,7 +11978,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K178" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L178" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -12022,7 +12022,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K179" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L179" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -12066,7 +12066,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K180" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L180" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -12110,7 +12110,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K181" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L181" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -12154,7 +12154,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K182" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L182" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -12198,7 +12198,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K183" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L183" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -12242,7 +12242,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K184" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L184" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -12286,7 +12286,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K185" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L185" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -12330,7 +12330,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K186" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.9672)</x:v>
       </x:c>
       <x:c r="L186" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -12374,7 +12374,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K187" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.9242)</x:v>
       </x:c>
       <x:c r="L187" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -12418,7 +12418,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K188" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L188" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -12462,7 +12462,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K189" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L189" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -12506,7 +12506,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K190" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.9180)</x:v>
       </x:c>
       <x:c r="L190" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -12550,7 +12550,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K191" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L191" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -12594,7 +12594,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K192" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.9167)</x:v>
       </x:c>
       <x:c r="L192" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -12638,7 +12638,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K193" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.9091)</x:v>
       </x:c>
       <x:c r="L193" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -12682,7 +12682,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K194" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.8974)</x:v>
       </x:c>
       <x:c r="L194" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -12726,7 +12726,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K195" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L195" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -12770,7 +12770,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K196" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L196" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -12814,7 +12814,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K197" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L197" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -12858,7 +12858,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K198" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.9701)</x:v>
       </x:c>
       <x:c r="L198" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -12902,7 +12902,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K199" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L199" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -12946,7 +12946,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K200" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L200" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -12990,7 +12990,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K201" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.9020)</x:v>
       </x:c>
       <x:c r="L201" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -13034,7 +13034,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K202" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L202" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -13078,7 +13078,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K203" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L203" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -13122,7 +13122,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K204" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L204" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -13166,7 +13166,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K205" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L205" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -13210,7 +13210,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K206" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L206" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -13254,7 +13254,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K207" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L207" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -13298,7 +13298,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K208" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L208" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -13342,7 +13342,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K209" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L209" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -13386,7 +13386,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K210" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.9565)</x:v>
       </x:c>
       <x:c r="L210" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -13430,7 +13430,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K211" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L211" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -13474,7 +13474,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K212" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L212" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -13518,7 +13518,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K213" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L213" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -13562,7 +13562,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K214" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L214" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -13606,7 +13606,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K215" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L215" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -13650,7 +13650,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K216" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L216" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -13694,7 +13694,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K217" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L217" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -13738,7 +13738,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K218" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L218" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -13782,7 +13782,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K219" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L219" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -13826,7 +13826,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K220" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L220" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -13870,7 +13870,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K221" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L221" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -13914,7 +13914,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K222" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.9394)</x:v>
       </x:c>
       <x:c r="L222" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -13958,7 +13958,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K223" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.9429)</x:v>
       </x:c>
       <x:c r="L223" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -14002,7 +14002,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K224" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L224" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -14046,7 +14046,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K225" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L225" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -14090,7 +14090,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K226" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L226" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -14134,7 +14134,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K227" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L227" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -14178,7 +14178,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K228" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L228" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -14222,7 +14222,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K229" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L229" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -14266,7 +14266,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K230" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L230" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -14310,7 +14310,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K231" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.9710)</x:v>
       </x:c>
       <x:c r="L231" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -14354,7 +14354,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K232" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L232" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -14398,7 +14398,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K233" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L233" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -14442,7 +14442,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K234" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L234" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -14486,7 +14486,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K235" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L235" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -14530,7 +14530,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K236" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L236" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -14574,7 +14574,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K237" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L237" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -14618,7 +14618,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K238" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L238" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -14662,7 +14662,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K239" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L239" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -14706,7 +14706,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K240" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.8857)</x:v>
       </x:c>
       <x:c r="L240" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -14750,7 +14750,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K241" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L241" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -14794,7 +14794,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K242" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L242" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -14838,7 +14838,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K243" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L243" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -14882,7 +14882,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K244" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L244" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -14926,7 +14926,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K245" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L245" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -14970,7 +14970,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K246" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L246" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -15014,7 +15014,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K247" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L247" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -15058,7 +15058,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K248" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L248" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -15102,7 +15102,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K249" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L249" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -15146,7 +15146,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K250" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L250" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -15190,7 +15190,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K251" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L251" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -15234,7 +15234,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K252" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L252" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -15278,7 +15278,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K253" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L253" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -15322,7 +15322,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K254" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L254" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -15366,7 +15366,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K255" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L255" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -15410,7 +15410,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K256" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L256" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -15454,7 +15454,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K257" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L257" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -15498,7 +15498,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K258" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L258" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -15542,7 +15542,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K259" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L259" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -15586,7 +15586,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K260" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L260" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -15630,7 +15630,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K261" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L261" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -15674,7 +15674,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K262" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L262" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -15718,7 +15718,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K263" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L263" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -15762,7 +15762,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K264" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L264" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -15806,7 +15806,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K265" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L265" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -15850,7 +15850,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K266" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L266" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -15894,7 +15894,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K267" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L267" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -15938,7 +15938,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K268" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L268" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -15982,7 +15982,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K269" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L269" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -16026,7 +16026,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K270" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L270" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -16070,7 +16070,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K271" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L271" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -16114,7 +16114,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K272" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.9286)</x:v>
       </x:c>
       <x:c r="L272" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -16158,7 +16158,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K273" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L273" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -16202,7 +16202,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K274" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L274" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -16246,7 +16246,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K275" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L275" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -16290,7 +16290,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K276" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L276" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -16334,7 +16334,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K277" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L277" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -16378,7 +16378,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K278" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L278" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -16422,7 +16422,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K279" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L279" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -16466,7 +16466,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K280" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L280" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -16510,7 +16510,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K281" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L281" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -16554,7 +16554,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K282" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L282" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -16598,7 +16598,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K283" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L283" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -16642,7 +16642,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K284" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L284" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -16686,7 +16686,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K285" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L285" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -16730,7 +16730,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K286" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L286" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -16774,7 +16774,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K287" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L287" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -16818,7 +16818,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K288" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L288" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -16862,7 +16862,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K289" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L289" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -16906,7 +16906,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K290" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L290" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -16950,7 +16950,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K291" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L291" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -16994,7 +16994,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K292" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.9583)</x:v>
       </x:c>
       <x:c r="L292" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -17038,7 +17038,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K293" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L293" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -17082,7 +17082,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K294" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L294" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -17126,7 +17126,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K295" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L295" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -17170,7 +17170,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K296" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.9595)</x:v>
       </x:c>
       <x:c r="L296" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -17214,7 +17214,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K297" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L297" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -17258,7 +17258,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K298" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L298" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -17302,7 +17302,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K299" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L299" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -17346,7 +17346,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K300" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.9492)</x:v>
       </x:c>
       <x:c r="L300" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -17390,7 +17390,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K301" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L301" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -17434,7 +17434,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K302" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L302" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -17478,7 +17478,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K303" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L303" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -17522,7 +17522,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K304" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L304" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -17566,7 +17566,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K305" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.9286)</x:v>
       </x:c>
       <x:c r="L305" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -17610,7 +17610,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K306" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L306" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -17654,7 +17654,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K307" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L307" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -17698,7 +17698,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K308" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.9552)</x:v>
       </x:c>
       <x:c r="L308" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -17742,7 +17742,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K309" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L309" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -17786,7 +17786,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K310" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.8718)</x:v>
       </x:c>
       <x:c r="L310" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -17830,7 +17830,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K311" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>OWNER LISTEN — long-form music identity is not inferred from its filename or speech transcription</x:v>
       </x:c>
       <x:c r="L311" s="21" t="str">
         <x:v>Measured: -15.99 LUFS integrated; -1.54 dBTP 4× estimate; -1.58 dBFS sample peak</x:v>
@@ -17874,7 +17874,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K312" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>OWNER LISTEN — long-form music identity is not inferred from its filename or speech transcription</x:v>
       </x:c>
       <x:c r="L312" s="21" t="str">
         <x:v>Measured: -12.72 LUFS integrated; 0.14 dBTP 4× estimate; 0 dBFS sample peak</x:v>
@@ -17918,7 +17918,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K313" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>OWNER LISTEN — long-form music identity is not inferred from its filename or speech transcription</x:v>
       </x:c>
       <x:c r="L313" s="21" t="str">
         <x:v>Measured: -14.05 LUFS integrated; -0.06 dBTP 4× estimate; -0.08 dBFS sample peak</x:v>
@@ -17962,7 +17962,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K314" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>OWNER LISTEN — long-form music identity is not inferred from its filename or speech transcription</x:v>
       </x:c>
       <x:c r="L314" s="21" t="str">
         <x:v>Measured: -16.37 LUFS integrated; -4.17 dBTP 4× estimate; -4.17 dBFS sample peak</x:v>
@@ -18006,7 +18006,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K315" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>OWNER LISTEN — long-form music identity is not inferred from its filename or speech transcription</x:v>
       </x:c>
       <x:c r="L315" s="21" t="str">
         <x:v>Measured: -12.21 LUFS integrated; 0.06 dBTP 4× estimate; 0 dBFS sample peak</x:v>
@@ -18050,7 +18050,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K316" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>OWNER LISTEN — long-form music identity is not inferred from its filename or speech transcription</x:v>
       </x:c>
       <x:c r="L316" s="21" t="str">
         <x:v>Measured: -11.23 LUFS integrated; -0.23 dBTP 4× estimate; -0.23 dBFS sample peak</x:v>
@@ -18094,7 +18094,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K317" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>OWNER LISTEN — long-form music identity is not inferred from its filename or speech transcription</x:v>
       </x:c>
       <x:c r="L317" s="21" t="str">
         <x:v>Measured: -10.04 LUFS integrated; 0.54 dBTP 4× estimate; 0.53 dBFS sample peak</x:v>
@@ -18138,7 +18138,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K318" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>OWNER LISTEN — long-form music identity is not inferred from its filename or speech transcription</x:v>
       </x:c>
       <x:c r="L318" s="21" t="str">
         <x:v>Measured: -13.15 LUFS integrated; 0.14 dBTP 4× estimate; 0.13 dBFS sample peak</x:v>
@@ -18182,7 +18182,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K319" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>OWNER LISTEN — long-form music identity is not inferred from its filename or speech transcription</x:v>
       </x:c>
       <x:c r="L319" s="21" t="str">
         <x:v>Measured: -14.68 LUFS integrated; -1.86 dBTP 4× estimate; -1.91 dBFS sample peak</x:v>
@@ -18226,7 +18226,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K320" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>OWNER LISTEN — long-form music identity is not inferred from its filename or speech transcription</x:v>
       </x:c>
       <x:c r="L320" s="21" t="str">
         <x:v>Measured: -11.22 LUFS integrated; 0 dBTP 4× estimate; 0 dBFS sample peak</x:v>
@@ -18270,7 +18270,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K321" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>OWNER LISTEN — long-form music identity is not inferred from its filename or speech transcription</x:v>
       </x:c>
       <x:c r="L321" s="21" t="str">
         <x:v>Measured: -13.46 LUFS integrated; -2.38 dBTP 4× estimate; -2.38 dBFS sample peak</x:v>
@@ -18314,7 +18314,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K322" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>OWNER LISTEN — long-form music identity is not inferred from its filename or speech transcription</x:v>
       </x:c>
       <x:c r="L322" s="21" t="str">
         <x:v>Measured: -15.73 LUFS integrated; -3.74 dBTP 4× estimate; -3.74 dBFS sample peak</x:v>
@@ -18346,28 +18346,28 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="G323" s="21" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H323" s="21" t="str">
-        <x:v>None found</x:v>
-      </x:c>
-      <x:c r="I323" s="23" t="str">
-        <x:v>YES — no source/runtime use found</x:v>
+        <x:v>apartment</x:v>
+      </x:c>
+      <x:c r="I323" s="21" t="str">
+        <x:v>No</x:v>
       </x:c>
       <x:c r="J323" s="21" t="str">
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K323" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.9716)</x:v>
       </x:c>
       <x:c r="L323" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M323" s="21" t="str">
-        <x:v>No reachable runtime use found</x:v>
+        <x:v>No source-level issue; active-play receipt pending</x:v>
       </x:c>
       <x:c r="N323" s="21" t="str">
-        <x:v>Mechanical: confirm the cue is dead, then remove the manifest row and file together; do not hide drift by renaming it.</x:v>
+        <x:v>Keep; verify audible content and loudness in the active scene.</x:v>
       </x:c>
     </x:row>
     <x:row r="324" ht="46" customHeight="1">
@@ -18390,28 +18390,28 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="G324" s="21" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H324" s="21" t="str">
-        <x:v>None found</x:v>
-      </x:c>
-      <x:c r="I324" s="23" t="str">
-        <x:v>YES — no source/runtime use found</x:v>
+        <x:v>apartment</x:v>
+      </x:c>
+      <x:c r="I324" s="21" t="str">
+        <x:v>No</x:v>
       </x:c>
       <x:c r="J324" s="21" t="str">
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K324" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L324" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M324" s="21" t="str">
-        <x:v>No reachable runtime use found</x:v>
+        <x:v>No source-level issue; active-play receipt pending</x:v>
       </x:c>
       <x:c r="N324" s="21" t="str">
-        <x:v>Mechanical: confirm the cue is dead, then remove the manifest row and file together; do not hide drift by renaming it.</x:v>
+        <x:v>Keep; verify audible content and loudness in the active scene.</x:v>
       </x:c>
     </x:row>
     <x:row r="325" ht="46" customHeight="1">
@@ -18434,28 +18434,28 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="G325" s="21" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H325" s="21" t="str">
-        <x:v>None found</x:v>
-      </x:c>
-      <x:c r="I325" s="23" t="str">
-        <x:v>YES — no source/runtime use found</x:v>
+        <x:v>apartment</x:v>
+      </x:c>
+      <x:c r="I325" s="21" t="str">
+        <x:v>No</x:v>
       </x:c>
       <x:c r="J325" s="21" t="str">
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K325" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L325" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M325" s="21" t="str">
-        <x:v>No reachable runtime use found</x:v>
+        <x:v>No source-level issue; active-play receipt pending</x:v>
       </x:c>
       <x:c r="N325" s="21" t="str">
-        <x:v>Mechanical: confirm the cue is dead, then remove the manifest row and file together; do not hide drift by renaming it.</x:v>
+        <x:v>Keep; verify audible content and loudness in the active scene.</x:v>
       </x:c>
     </x:row>
     <x:row r="326" ht="46" customHeight="1">
@@ -18478,28 +18478,28 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="G326" s="21" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H326" s="21" t="str">
-        <x:v>None found</x:v>
-      </x:c>
-      <x:c r="I326" s="23" t="str">
-        <x:v>YES — no source/runtime use found</x:v>
+        <x:v>apartment</x:v>
+      </x:c>
+      <x:c r="I326" s="21" t="str">
+        <x:v>No</x:v>
       </x:c>
       <x:c r="J326" s="21" t="str">
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K326" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L326" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M326" s="21" t="str">
-        <x:v>No reachable runtime use found</x:v>
+        <x:v>No source-level issue; active-play receipt pending</x:v>
       </x:c>
       <x:c r="N326" s="21" t="str">
-        <x:v>Mechanical: confirm the cue is dead, then remove the manifest row and file together; do not hide drift by renaming it.</x:v>
+        <x:v>Keep; verify audible content and loudness in the active scene.</x:v>
       </x:c>
     </x:row>
     <x:row r="327" ht="46" customHeight="1">
@@ -18522,28 +18522,28 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="G327" s="21" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H327" s="21" t="str">
-        <x:v>None found</x:v>
-      </x:c>
-      <x:c r="I327" s="23" t="str">
-        <x:v>YES — no source/runtime use found</x:v>
+        <x:v>apartment</x:v>
+      </x:c>
+      <x:c r="I327" s="21" t="str">
+        <x:v>No</x:v>
       </x:c>
       <x:c r="J327" s="21" t="str">
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K327" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L327" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M327" s="21" t="str">
-        <x:v>No reachable runtime use found</x:v>
+        <x:v>No source-level issue; active-play receipt pending</x:v>
       </x:c>
       <x:c r="N327" s="21" t="str">
-        <x:v>Mechanical: confirm the cue is dead, then remove the manifest row and file together; do not hide drift by renaming it.</x:v>
+        <x:v>Keep; verify audible content and loudness in the active scene.</x:v>
       </x:c>
     </x:row>
     <x:row r="328" ht="46" customHeight="1">
@@ -18566,28 +18566,28 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="G328" s="21" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H328" s="21" t="str">
-        <x:v>None found</x:v>
-      </x:c>
-      <x:c r="I328" s="23" t="str">
-        <x:v>YES — no source/runtime use found</x:v>
+        <x:v>apartment</x:v>
+      </x:c>
+      <x:c r="I328" s="21" t="str">
+        <x:v>No</x:v>
       </x:c>
       <x:c r="J328" s="21" t="str">
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K328" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L328" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M328" s="21" t="str">
-        <x:v>No reachable runtime use found</x:v>
+        <x:v>No source-level issue; active-play receipt pending</x:v>
       </x:c>
       <x:c r="N328" s="21" t="str">
-        <x:v>Mechanical: confirm the cue is dead, then remove the manifest row and file together; do not hide drift by renaming it.</x:v>
+        <x:v>Keep; verify audible content and loudness in the active scene.</x:v>
       </x:c>
     </x:row>
     <x:row r="329" ht="46" customHeight="1">
@@ -18610,28 +18610,28 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="G329" s="21" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H329" s="21" t="str">
-        <x:v>None found</x:v>
-      </x:c>
-      <x:c r="I329" s="23" t="str">
-        <x:v>YES — no source/runtime use found</x:v>
+        <x:v>apartment</x:v>
+      </x:c>
+      <x:c r="I329" s="21" t="str">
+        <x:v>No</x:v>
       </x:c>
       <x:c r="J329" s="21" t="str">
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K329" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L329" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M329" s="21" t="str">
-        <x:v>No reachable runtime use found</x:v>
+        <x:v>No source-level issue; active-play receipt pending</x:v>
       </x:c>
       <x:c r="N329" s="21" t="str">
-        <x:v>Mechanical: confirm the cue is dead, then remove the manifest row and file together; do not hide drift by renaming it.</x:v>
+        <x:v>Keep; verify audible content and loudness in the active scene.</x:v>
       </x:c>
     </x:row>
     <x:row r="330" ht="46" customHeight="1">
@@ -18654,28 +18654,28 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="G330" s="21" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H330" s="21" t="str">
-        <x:v>None found</x:v>
-      </x:c>
-      <x:c r="I330" s="23" t="str">
-        <x:v>YES — no source/runtime use found</x:v>
+        <x:v>apartment</x:v>
+      </x:c>
+      <x:c r="I330" s="21" t="str">
+        <x:v>No</x:v>
       </x:c>
       <x:c r="J330" s="21" t="str">
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K330" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L330" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M330" s="21" t="str">
-        <x:v>No reachable runtime use found</x:v>
+        <x:v>No source-level issue; active-play receipt pending</x:v>
       </x:c>
       <x:c r="N330" s="21" t="str">
-        <x:v>Mechanical: confirm the cue is dead, then remove the manifest row and file together; do not hide drift by renaming it.</x:v>
+        <x:v>Keep; verify audible content and loudness in the active scene.</x:v>
       </x:c>
     </x:row>
     <x:row r="331" ht="46" customHeight="1">
@@ -18698,28 +18698,28 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="G331" s="21" t="n">
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="H331" s="21" t="str">
-        <x:v>None found</x:v>
-      </x:c>
-      <x:c r="I331" s="23" t="str">
-        <x:v>YES — no source/runtime use found</x:v>
+        <x:v>apartment</x:v>
+      </x:c>
+      <x:c r="I331" s="21" t="str">
+        <x:v>No</x:v>
       </x:c>
       <x:c r="J331" s="21" t="str">
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K331" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L331" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M331" s="21" t="str">
-        <x:v>No reachable runtime use found</x:v>
+        <x:v>No source-level issue; active-play receipt pending</x:v>
       </x:c>
       <x:c r="N331" s="21" t="str">
-        <x:v>Mechanical: confirm the cue is dead, then remove the manifest row and file together; do not hide drift by renaming it.</x:v>
+        <x:v>Keep; verify audible content and loudness in the active scene.</x:v>
       </x:c>
     </x:row>
     <x:row r="332" ht="46" customHeight="1">
@@ -18742,28 +18742,28 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="G332" s="21" t="n">
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H332" s="21" t="str">
-        <x:v>None found</x:v>
-      </x:c>
-      <x:c r="I332" s="23" t="str">
-        <x:v>YES — no source/runtime use found</x:v>
+        <x:v>apartment</x:v>
+      </x:c>
+      <x:c r="I332" s="21" t="str">
+        <x:v>No</x:v>
       </x:c>
       <x:c r="J332" s="21" t="str">
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K332" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L332" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
       </x:c>
       <x:c r="M332" s="21" t="str">
-        <x:v>No reachable runtime use found</x:v>
+        <x:v>No source-level issue; active-play receipt pending</x:v>
       </x:c>
       <x:c r="N332" s="21" t="str">
-        <x:v>Mechanical: confirm the cue is dead, then remove the manifest row and file together; do not hide drift by renaming it.</x:v>
+        <x:v>Keep; verify audible content and loudness in the active scene.</x:v>
       </x:c>
     </x:row>
     <x:row r="333" ht="46" customHeight="1">
@@ -18798,7 +18798,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K333" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L333" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -18842,7 +18842,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K334" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L334" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -18886,7 +18886,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K335" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L335" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -18930,7 +18930,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K336" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.9535)</x:v>
       </x:c>
       <x:c r="L336" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -18974,7 +18974,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K337" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L337" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -19018,7 +19018,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K338" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L338" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -19062,7 +19062,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K339" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L339" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -19106,7 +19106,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K340" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L340" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -19150,7 +19150,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K341" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L341" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -19194,7 +19194,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K342" s="21" t="str">
-        <x:v>UNVERIFIED — manifest text/title is not an audio-content check</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
       </x:c>
       <x:c r="L342" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -19214,7 +19214,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b307329418845a1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R638a194acb504564"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19265,7 +19265,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="10" t="str">
-        <x:v>13 data rows · Generated by tools/radio-audit.mjs · Source-only findings remain explicitly marked for active-play/loudness/content verification.</x:v>
+        <x:v>13 data rows · Generated by tools/radio-audit.mjs · Active-play mix, music identity, provenance, and owner decisions remain explicitly marked.</x:v>
       </x:c>
       <x:c r="B3" s="10"/>
       <x:c r="C3" s="10"/>
@@ -19320,16 +19320,16 @@
         <x:v>Station architecture</x:v>
       </x:c>
       <x:c r="D6" s="24" t="str">
-        <x:v>The station source comment still documents three selectable stations, but STATIONS exports one live station.</x:v>
+        <x:v>Runtime and source documentation now agree that 97.8 THE SQUATCH is the one live station; `uncle` and `ksqch` remain unresolved legacy identities only.</x:v>
       </x:c>
       <x:c r="E6" s="24" t="str">
         <x:v>src/core/stations.js:4</x:v>
       </x:c>
       <x:c r="F6" s="24" t="str">
-        <x:v>No direct runtime failure; developers can make wrong playlist and UI assumptions.</x:v>
+        <x:v>Resolved for current development: agents no longer mistake legacy tags for selectable dials.</x:v>
       </x:c>
       <x:c r="G6" s="24" t="str">
-        <x:v>Mechanical: update the comment after the owner decides whether the two legacy identities are retired or returning.</x:v>
+        <x:v>Documentation is corrected. Do not revive or delete legacy identities until the owner decides their future.</x:v>
       </x:c>
       <x:c r="H6" s="24" t="str">
         <x:v>Mechanical</x:v>
@@ -19338,7 +19338,7 @@
         <x:v>OWNER: retire or restore `uncle` and `ksqch` identities.</x:v>
       </x:c>
       <x:c r="J6" s="24" t="str">
-        <x:v>OPEN</x:v>
+        <x:v>DOCUMENTED — OWNER DECISION OPEN</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="54" customHeight="1">
@@ -19352,16 +19352,16 @@
         <x:v>assets/music/manifest.json `station`</x:v>
       </x:c>
       <x:c r="D7" s="24" t="str">
-        <x:v>The manifest says `station` assigns dial position; Radio.playlist ignores `station` and filters only `cue` plus exact `venue`.</x:v>
+        <x:v>The manifest now labels `station` as ignored legacy catalog metadata; current Radio.playlist intentionally filters only `cue` plus exact `venue`.</x:v>
       </x:c>
       <x:c r="E7" s="24" t="str">
-        <x:v>assets/music/manifest.json:2 vs src/core/radio.js:201</x:v>
+        <x:v>assets/music/manifest.json:2 and src/core/radio.js:201</x:v>
       </x:c>
       <x:c r="F7" s="24" t="str">
-        <x:v>Legacy-tagged unscoped records can air on 97.8 in every physical receiver.</x:v>
+        <x:v>Current behavior is documented: legacy-tagged unscoped records can air on 97.8 in every physical receiver.</x:v>
       </x:c>
       <x:c r="G7" s="24" t="str">
-        <x:v>Mechanical after OWNER decision: reconcile manifest metadata with actual selection logic and add a contract test.</x:v>
+        <x:v>After OWNER decides station/venue allocation, update metadata and runtime together with a contract test.</x:v>
       </x:c>
       <x:c r="H7" s="24" t="str">
         <x:v>Mechanical</x:v>
@@ -19370,7 +19370,7 @@
         <x:v>OWNER: desired station/venue allocation for existing tracks.</x:v>
       </x:c>
       <x:c r="J7" s="24" t="str">
-        <x:v>OPEN</x:v>
+        <x:v>DOCUMENTED — OWNER DECISION OPEN</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="54" customHeight="1">
@@ -19384,25 +19384,25 @@
         <x:v>Physical 97.8 receivers</x:v>
       </x:c>
       <x:c r="D8" s="22" t="str">
-        <x:v>These receiver implementations do not use createCampaignRadioAdapter while the apartment, cabin, Bing car, Beef Run, No Wake, and golf cart do.</x:v>
+        <x:v>Luxury Apartment and both Mansion visits previously reset their physical 97.8 receivers instead of using the shared campaign adapter.</x:v>
       </x:c>
       <x:c r="E8" s="22" t="str">
-        <x:v>src/luxury-apartment/main.js:299; src/mansion/main.js:846</x:v>
+        <x:v>src/luxury-apartment/main.js:302; src/mansion/main.js:856; focused residency and real-browser reload receipts.</x:v>
       </x:c>
       <x:c r="F8" s="22" t="str">
-        <x:v>Power, volume, cursor, and selection continuity reset on reload or scene return.</x:v>
+        <x:v>Resolved: saved power, volume, cursor, and selection now survive reload without autoplay before the player gesture or duplicate Mansion talk beds.</x:v>
       </x:c>
       <x:c r="G8" s="22" t="str">
-        <x:v>Mechanical: add unique receiver IDs and the shared adapter if those radios should follow campaign continuity.</x:v>
+        <x:v>Implemented: unique Luxury ownership and one shared physical Mansion house tuner, both default-off and restored after audio unlock.</x:v>
       </x:c>
       <x:c r="H8" s="22" t="str">
         <x:v>Mechanical</x:v>
       </x:c>
       <x:c r="I8" s="22" t="str">
-        <x:v>No; use the established shared receiver behavior.</x:v>
+        <x:v>No; used the established shared receiver behavior.</x:v>
       </x:c>
       <x:c r="J8" s="22" t="str">
-        <x:v>OPEN</x:v>
+        <x:v>RESOLVED</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="54" customHeight="1">
@@ -19608,7 +19608,7 @@
         <x:v>Cue inventory</x:v>
       </x:c>
       <x:c r="D15" s="24" t="str">
-        <x:v>14 radio/music assets have no reachable source/runtime use; 0 referenced audit assets are missing.</x:v>
+        <x:v>4 radio/music assets have no reachable source/runtime use; 0 referenced audit assets are missing.</x:v>
       </x:c>
       <x:c r="E15" s="24" t="str">
         <x:v>Generated Cue Inventory combines manifests, generated voice cue names, source references, receiver eligibility, and byte hashes.</x:v>
@@ -19630,35 +19630,35 @@
       </x:c>
     </x:row>
     <x:row r="16" ht="54" customHeight="1">
-      <x:c r="A16" s="21" t="str">
+      <x:c r="A16" s="24" t="str">
         <x:v>P2</x:v>
       </x:c>
-      <x:c r="B16" s="21" t="str">
+      <x:c r="B16" s="24" t="str">
         <x:v>Global</x:v>
       </x:c>
-      <x:c r="C16" s="21" t="str">
+      <x:c r="C16" s="24" t="str">
         <x:v>Filename/content and source-only audit limit</x:v>
       </x:c>
-      <x:c r="D16" s="21" t="str">
-        <x:v>A filename, manifest title, or current cue text does not prove the recording actually contains that content.</x:v>
-      </x:c>
-      <x:c r="E16" s="21" t="str">
-        <x:v>Every Cue Inventory row marks audio identity UNVERIFIED; no transcription/listening comparison is part of the current generator.</x:v>
-      </x:c>
-      <x:c r="F16" s="21" t="str">
-        <x:v>A correctly named but stale/wrong take can pass source checks.</x:v>
-      </x:c>
-      <x:c r="G16" s="21" t="str">
-        <x:v>Mechanical: add transcription or supervised listening comparison and record exceptions explicitly.</x:v>
-      </x:c>
-      <x:c r="H16" s="21" t="str">
+      <x:c r="D16" s="24" t="str">
+        <x:v>298 spoken station/news cues have current hash-bound Scribe v2 receipts; 0 spoken cues remain stale, missing, or below the review threshold. Long-form music still requires owner listening/provenance.</x:v>
+      </x:c>
+      <x:c r="E16" s="24" t="str">
+        <x:v>docs/audits/radio/content-transcriptions.json binds cue, current authored text hash, voice, delivered MP3 hash, transcript, language, and similarity.</x:v>
+      </x:c>
+      <x:c r="F16" s="24" t="str">
+        <x:v>A correctly named but stale/wrong spoken take now fails the content gate; music identity is still explicitly not inferred from filenames.</x:v>
+      </x:c>
+      <x:c r="G16" s="24" t="str">
+        <x:v>Mechanical spoken-content verification is implemented. OWNER supplies provenance and reviews retained music identity; rerender any future speech review row.</x:v>
+      </x:c>
+      <x:c r="H16" s="24" t="str">
         <x:v>Mechanical</x:v>
       </x:c>
-      <x:c r="I16" s="21" t="str">
-        <x:v>No for detection; OWNER resolves creative mismatches.</x:v>
-      </x:c>
-      <x:c r="J16" s="21" t="str">
-        <x:v>OPEN</x:v>
+      <x:c r="I16" s="24" t="str">
+        <x:v>OWNER only for long-form music provenance/identity or a genuine creative speech mismatch.</x:v>
+      </x:c>
+      <x:c r="J16" s="24" t="str">
+        <x:v>RESOLVED FOR SPOKEN CUES — MUSIC OWNER REVIEW</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="54" customHeight="1">
@@ -19733,7 +19733,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcbd978e9baec47d0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8cf792fed884834"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19778,7 +19778,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="10" t="str">
-        <x:v>9 data rows · Generated by tools/radio-audit.mjs · Source-only findings remain explicitly marked for active-play/loudness/content verification.</x:v>
+        <x:v>9 data rows · Generated by tools/radio-audit.mjs · Active-play mix, music identity, provenance, and owner decisions remain explicitly marked.</x:v>
       </x:c>
       <x:c r="B3" s="10"/>
       <x:c r="C3" s="10"/>
@@ -19845,48 +19845,50 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B7" s="24" t="str">
-        <x:v>Reconcile stale station comments and manifest semantics</x:v>
+        <x:v>Reconcile station documentation and manifest semantics while preserving unresolved legacy identities</x:v>
       </x:c>
       <x:c r="C7" s="24" t="str">
         <x:v>src/core/stations.js; assets/music/manifest.json; src/core/radio.js; tests/radio-*.test.mjs</x:v>
       </x:c>
       <x:c r="D7" s="24" t="str">
-        <x:v>OWNER rules on legacy uncle/ksqch identities</x:v>
+        <x:v>OWNER rules on legacy uncle/ksqch identities for any runtime change</x:v>
       </x:c>
       <x:c r="E7" s="24" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="F7" s="24" t="str">
-        <x:v>Docs, manifest, runtime selection, and tests describe the same station model</x:v>
+        <x:v>Docs, manifest, runtime selection, and tests describe the same current station model without guessing the legacy identities future</x:v>
       </x:c>
       <x:c r="G7" s="24" t="str">
-        <x:v>WAITING ON OWNER</x:v>
+        <x:v>DOCUMENTATION DONE — IDENTITY DECISION OWNER</x:v>
       </x:c>
       <x:c r="H7" s="24" t="str"/>
     </x:row>
     <x:row r="8" ht="54" customHeight="1">
-      <x:c r="A8" s="21" t="n">
+      <x:c r="A8" s="25" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B8" s="21" t="str">
+      <x:c r="B8" s="25" t="str">
         <x:v>Make receiver persistence consistent</x:v>
       </x:c>
-      <x:c r="C8" s="21" t="str">
+      <x:c r="C8" s="25" t="str">
         <x:v>src/luxury-apartment/main.js; src/mansion/main.js; src/core/campaign.js</x:v>
       </x:c>
-      <x:c r="D8" s="21" t="str">
+      <x:c r="D8" s="25" t="str">
         <x:v>Existing createCampaignRadioAdapter</x:v>
       </x:c>
-      <x:c r="E8" s="21" t="str">
+      <x:c r="E8" s="25" t="str">
         <x:v>Low</x:v>
       </x:c>
-      <x:c r="F8" s="21" t="str">
+      <x:c r="F8" s="25" t="str">
         <x:v>Power, volume, cursor, and selection survive reload without cross-receiver collisions</x:v>
       </x:c>
-      <x:c r="G8" s="21" t="str">
-        <x:v>READY</x:v>
-      </x:c>
-      <x:c r="H8" s="21" t="str"/>
+      <x:c r="G8" s="25" t="str">
+        <x:v>DONE</x:v>
+      </x:c>
+      <x:c r="H8" s="25" t="str">
+        <x:v>4d7d01ef</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="54" customHeight="1">
       <x:c r="A9" s="21" t="n">
@@ -19908,33 +19910,35 @@
         <x:v>Each changed scene proves active keys, stops, reload state, console errors, and no unintended concurrent masters</x:v>
       </x:c>
       <x:c r="G9" s="21" t="str">
-        <x:v>READY</x:v>
-      </x:c>
-      <x:c r="H9" s="21" t="str"/>
+        <x:v>HOME RECEIVER RECEIPTS DONE — CAMPAIGN MIX PASS OPEN</x:v>
+      </x:c>
+      <x:c r="H9" s="21" t="str">
+        <x:v>4d7d01ef</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="54" customHeight="1">
-      <x:c r="A10" s="21" t="n">
+      <x:c r="A10" s="24" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B10" s="21" t="str">
+      <x:c r="B10" s="24" t="str">
         <x:v>Add repeatable duration, integrated-loudness, true-peak, and identity evidence</x:v>
       </x:c>
-      <x:c r="C10" s="21" t="str">
-        <x:v>tools/audio-loudness-audit.mjs; docs/audits/radio/loudness-measurements.json; tools/radio-audit.mjs; generated Cue Inventory</x:v>
-      </x:c>
-      <x:c r="D10" s="21" t="str">
-        <x:v>Existing Playwright Chromium decoder; supervised listening/transcription for content identity</x:v>
-      </x:c>
-      <x:c r="E10" s="21" t="str">
+      <x:c r="C10" s="24" t="str">
+        <x:v>tools/audio-loudness-audit.mjs; tools/verify-radio-content.ps1; docs/audits/radio/loudness-measurements.json; docs/audits/radio/content-transcriptions.json; tools/radio-audit.mjs; generated Cue Inventory</x:v>
+      </x:c>
+      <x:c r="D10" s="24" t="str">
+        <x:v>Existing Playwright Chromium decoder and ElevenLabs Scribe v2 for spoken identity</x:v>
+      </x:c>
+      <x:c r="E10" s="24" t="str">
         <x:v>Medium</x:v>
       </x:c>
-      <x:c r="F10" s="21" t="str">
-        <x:v>Every retained master has measured duration/LUFS/peak and verified content or an explicit exception</x:v>
-      </x:c>
-      <x:c r="G10" s="21" t="str">
-        <x:v>LOUDNESS DONE — CONTENT IDENTITY PENDING</x:v>
-      </x:c>
-      <x:c r="H10" s="21" t="str"/>
+      <x:c r="F10" s="24" t="str">
+        <x:v>Every retained master has measured duration/LUFS/peak; every spoken cue has a current transcript; music identity remains an explicit owner review</x:v>
+      </x:c>
+      <x:c r="G10" s="24" t="str">
+        <x:v>LOUDNESS + SPOKEN IDENTITY DONE — MUSIC OWNER REVIEW</x:v>
+      </x:c>
+      <x:c r="H10" s="24" t="str"/>
     </x:row>
     <x:row r="11" ht="54" customHeight="1">
       <x:c r="A11" s="24" t="n">
@@ -19961,28 +19965,30 @@
       <x:c r="H11" s="24" t="str"/>
     </x:row>
     <x:row r="12" ht="54" customHeight="1">
-      <x:c r="A12" s="21" t="n">
+      <x:c r="A12" s="24" t="n">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B12" s="21" t="str">
+      <x:c r="B12" s="24" t="str">
         <x:v>Implement approved mechanical trigger, stop, restore, and selection fixes</x:v>
       </x:c>
-      <x:c r="C12" s="21" t="str">
+      <x:c r="C12" s="24" t="str">
         <x:v>src/core/radio.js; scene-owned score modules; manifests; relevant tests</x:v>
       </x:c>
-      <x:c r="D12" s="21" t="str">
+      <x:c r="D12" s="24" t="str">
         <x:v>Orders 2–6</x:v>
       </x:c>
-      <x:c r="E12" s="21" t="str">
+      <x:c r="E12" s="24" t="str">
         <x:v>Medium</x:v>
       </x:c>
-      <x:c r="F12" s="21" t="str">
+      <x:c r="F12" s="24" t="str">
         <x:v>Source contracts and real-browser receipts pass; owner-selected material remains intact</x:v>
       </x:c>
-      <x:c r="G12" s="21" t="str">
-        <x:v>BLOCKED BY DECISIONS/EVIDENCE</x:v>
-      </x:c>
-      <x:c r="H12" s="21" t="str"/>
+      <x:c r="G12" s="24" t="str">
+        <x:v>HOME RECEIVER FIX DONE — PROGRAMMING CHANGES WAIT ON OWNER</x:v>
+      </x:c>
+      <x:c r="H12" s="24" t="str">
+        <x:v>4d7d01ef</x:v>
+      </x:c>
     </x:row>
     <x:row r="13" ht="54" customHeight="1">
       <x:c r="A13" s="21" t="n">
@@ -20040,7 +20046,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ad5707d6a9f4ad8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37d9340fa7e840c1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
ci(evidence): gate radio and rendered voices
Make the 386-render browser receipts, generated radio audit, 24-master loudness ledger, and 298 spoken-content transcripts part of the authoritative pull-request workflow. Add discoverable package commands and push-card guidance, and stamp the generated radio revamp plan with the commits that supplied its evidence. Local package-command checks, audit drift checks, workbook QA (5 sheets, zero formula errors), and diff checks passed.
</commit_message>
<xml_diff>
--- a/docs/audits/SQUATCHSMASH-RADIO-AUDIT.xlsx
+++ b/docs/audits/SQUATCHSMASH-RADIO-AUDIT.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scene Timeline" sheetId="1" r:id="R36b1b4ba8b8e4009"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Station Catalog" sheetId="2" r:id="R5b92ed2b17a746bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cue Inventory" sheetId="3" r:id="R0d5cf8d5b2924182"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Problems and Decisions" sheetId="4" r:id="R8887422464b24d46"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revamp Plan" sheetId="5" r:id="Rbf6b0c7f8d9d450a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scene Timeline" sheetId="1" r:id="R2da9fc86ec404a7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Station Catalog" sheetId="2" r:id="Re8bbbe514ff84cab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cue Inventory" sheetId="3" r:id="Ra5665527edef4586"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Problems and Decisions" sheetId="4" r:id="R5bcdab4e71e94916"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revamp Plan" sheetId="5" r:id="Rbceffc5897014e4b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4008,7 +4008,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re332e63e7a9e4173"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa04686527b94de5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4255,7 +4255,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4758d816acb74388"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcbb9472a87a04164"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19214,7 +19214,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R638a194acb504564"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ac2dd538881477b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19733,7 +19733,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8cf792fed884834"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a1fb3e674ae42ce"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19837,7 +19837,7 @@
         <x:v>DONE</x:v>
       </x:c>
       <x:c r="H6" s="25" t="str">
-        <x:v>This audit commit</x:v>
+        <x:v>d6f2ae0e; b2e63abb</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="54" customHeight="1">
@@ -19862,7 +19862,9 @@
       <x:c r="G7" s="24" t="str">
         <x:v>DOCUMENTATION DONE — IDENTITY DECISION OWNER</x:v>
       </x:c>
-      <x:c r="H7" s="24" t="str"/>
+      <x:c r="H7" s="24" t="str">
+        <x:v>b2e63abb</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="54" customHeight="1">
       <x:c r="A8" s="25" t="n">
@@ -19938,7 +19940,9 @@
       <x:c r="G10" s="24" t="str">
         <x:v>LOUDNESS + SPOKEN IDENTITY DONE — MUSIC OWNER REVIEW</x:v>
       </x:c>
-      <x:c r="H10" s="24" t="str"/>
+      <x:c r="H10" s="24" t="str">
+        <x:v>14cc6c94; b2e63abb</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="54" customHeight="1">
       <x:c r="A11" s="24" t="n">
@@ -20046,7 +20050,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37d9340fa7e840c1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5016e2906204849"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
chore(audio): finalize voices and campaign radio ledger
</commit_message>
<xml_diff>
--- a/docs/audits/SQUATCHSMASH-RADIO-AUDIT.xlsx
+++ b/docs/audits/SQUATCHSMASH-RADIO-AUDIT.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scene Timeline" sheetId="1" r:id="R2da9fc86ec404a7b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Station Catalog" sheetId="2" r:id="Re8bbbe514ff84cab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cue Inventory" sheetId="3" r:id="Ra5665527edef4586"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Problems and Decisions" sheetId="4" r:id="R5bcdab4e71e94916"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revamp Plan" sheetId="5" r:id="Rbceffc5897014e4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scene Timeline" sheetId="1" r:id="Rd8458af365ea46fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Station Catalog" sheetId="2" r:id="Rd6a14db59df949f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cue Inventory" sheetId="3" r:id="R8e33e96cc81b4d5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Problems and Decisions" sheetId="4" r:id="R613924a8d9854b64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revamp Plan" sheetId="5" r:id="R4da513ee20e34b3d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1932,7 +1932,7 @@
         <x:v>Day 5</x:v>
       </x:c>
       <x:c r="D22" s="21" t="str">
-        <x:v>01:30–04:30 anchored mission window</x:v>
+        <x:v>01:30–06:30 overnight cover window; incident resolves before Snow’s daylight drop</x:v>
       </x:c>
       <x:c r="E22" s="21" t="str">
         <x:v>jerky_motel</x:v>
@@ -3164,7 +3164,7 @@
         <x:v>Day 8–9</x:v>
       </x:c>
       <x:c r="D38" s="21" t="str">
-        <x:v>Mansion evening then eight-hour guest-room rest</x:v>
+        <x:v>Mansion evening then six-hour guest-room rest</x:v>
       </x:c>
       <x:c r="E38" s="21" t="str">
         <x:v>mansion</x:v>
@@ -3312,7 +3312,7 @@
         <x:v>war</x:v>
       </x:c>
       <x:c r="B40" s="21" t="str">
-        <x:v>24 · Enola Squatch</x:v>
+        <x:v>24 · SQUATCHOLA GAY</x:v>
       </x:c>
       <x:c r="C40" s="21" t="str">
         <x:v>Day 9</x:v>
@@ -3389,7 +3389,7 @@
         <x:v>war</x:v>
       </x:c>
       <x:c r="B41" s="21" t="str">
-        <x:v>24 · Enola Squatch</x:v>
+        <x:v>24 · SQUATCHOLA GAY</x:v>
       </x:c>
       <x:c r="C41" s="21" t="str">
         <x:v>Day 9</x:v>
@@ -3466,7 +3466,7 @@
         <x:v>war</x:v>
       </x:c>
       <x:c r="B42" s="21" t="str">
-        <x:v>24 · Enola Squatch</x:v>
+        <x:v>24 · SQUATCHOLA GAY</x:v>
       </x:c>
       <x:c r="C42" s="21" t="str">
         <x:v>Day 9</x:v>
@@ -3543,7 +3543,7 @@
         <x:v>war</x:v>
       </x:c>
       <x:c r="B43" s="21" t="str">
-        <x:v>24 · Enola Squatch</x:v>
+        <x:v>24 · SQUATCHOLA GAY</x:v>
       </x:c>
       <x:c r="C43" s="21" t="str">
         <x:v>Day 9</x:v>
@@ -4008,7 +4008,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa04686527b94de5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb04dfb5770724c08"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4255,7 +4255,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcbb9472a87a04164"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R13226df72c554166"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4700,7 +4700,7 @@
         <x:v>232.046</x:v>
       </x:c>
       <x:c r="E13" s="21" t="str">
-        <x:v>Artist metadata: Creedence Clearwater Revival. The Enola Squatch's takeoff needle-drop, same mechanism as Beef Run's. No station and no venue -- a cue, not programming. Runtime reads MissionAudio.takeoffAnthemFile in src/beefrun/audio.js, set in src/enolasquatch/main.js. License/source field not recorded in manifest.</x:v>
+        <x:v>Artist metadata: Creedence Clearwater Revival. SQUATCHOLA GAY's takeoff needle-drop, same mechanism as Beef Run's. No station and no venue -- a cue, not programming. Runtime reads MissionAudio.takeoffAnthemFile in src/beefrun/audio.js, set in src/enolasquatch/main.js. License/source field not recorded in manifest.</x:v>
       </x:c>
       <x:c r="F13" s="21" t="str">
         <x:v>No</x:v>
@@ -8912,16 +8912,16 @@
     </x:row>
     <x:row r="109" ht="46" customHeight="1">
       <x:c r="A109" s="21" t="str">
-        <x:v>radio.vo.announcer.157erj5</x:v>
+        <x:v>radio.vo.announcer.15n90um</x:v>
       </x:c>
       <x:c r="B109" s="21" t="str">
-        <x:v>assets/sfx/radio.vo.announcer.157erj5.mp3</x:v>
+        <x:v>assets/sfx/radio.vo.announcer.15n90um.mp3</x:v>
       </x:c>
       <x:c r="C109" s="21" t="str">
         <x:v>MP3</x:v>
       </x:c>
       <x:c r="D109" s="21" t="n">
-        <x:v>4.049</x:v>
+        <x:v>8.568</x:v>
       </x:c>
       <x:c r="E109" s="21" t="str">
         <x:v>Voice: announcer. License/source field not recorded in manifest.</x:v>
@@ -8956,16 +8956,16 @@
     </x:row>
     <x:row r="110" ht="46" customHeight="1">
       <x:c r="A110" s="21" t="str">
-        <x:v>radio.vo.announcer.15n90um</x:v>
+        <x:v>radio.vo.announcer.170fb70</x:v>
       </x:c>
       <x:c r="B110" s="21" t="str">
-        <x:v>assets/sfx/radio.vo.announcer.15n90um.mp3</x:v>
+        <x:v>assets/sfx/radio.vo.announcer.170fb70.mp3</x:v>
       </x:c>
       <x:c r="C110" s="21" t="str">
         <x:v>MP3</x:v>
       </x:c>
       <x:c r="D110" s="21" t="n">
-        <x:v>8.568</x:v>
+        <x:v>9.117</x:v>
       </x:c>
       <x:c r="E110" s="21" t="str">
         <x:v>Voice: announcer. License/source field not recorded in manifest.</x:v>
@@ -8986,7 +8986,7 @@
         <x:v>No byte-identical audit duplicate</x:v>
       </x:c>
       <x:c r="K110" s="21" t="str">
-        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (1.0000)</x:v>
+        <x:v>VERIFIED — hash-bound Scribe v2 transcript matches authored speech (0.9909)</x:v>
       </x:c>
       <x:c r="L110" s="21" t="str">
         <x:v>Not a long-form master — excluded from the music-master loudness pass; active speech/effect mix receipt pending</x:v>
@@ -19214,7 +19214,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ac2dd538881477b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e765472ebd1484f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19547,7 +19547,7 @@
         <x:v>Mission-aware NEWS_SEGMENTS are enabled on the apartment and cabin receivers only; other receivers run the same station without news eligibility.</x:v>
       </x:c>
       <x:c r="E13" s="24" t="str">
-        <x:v>src/main.js:427; src/cabin/main.js:167</x:v>
+        <x:v>src/main.js:427; src/cabin/main.js:169</x:v>
       </x:c>
       <x:c r="F13" s="24" t="str">
         <x:v>A player can hear the same station in another location but not the campaign bulletin that is eligible at home.</x:v>
@@ -19733,7 +19733,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a1fb3e674ae42ce"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0236f3613bcb4304"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20050,7 +20050,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5016e2906204849"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R25cf4287518b46f4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
test(audio): close campaign radio lifecycle coverage
</commit_message>
<xml_diff>
--- a/docs/audits/SQUATCHSMASH-RADIO-AUDIT.xlsx
+++ b/docs/audits/SQUATCHSMASH-RADIO-AUDIT.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scene Timeline" sheetId="1" r:id="Rd8458af365ea46fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Station Catalog" sheetId="2" r:id="Rd6a14db59df949f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cue Inventory" sheetId="3" r:id="R8e33e96cc81b4d5d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Problems and Decisions" sheetId="4" r:id="R613924a8d9854b64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revamp Plan" sheetId="5" r:id="R4da513ee20e34b3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scene Timeline" sheetId="1" r:id="R56b92b7bce5b4e7d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Station Catalog" sheetId="2" r:id="R13a59ddfeee34914"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cue Inventory" sheetId="3" r:id="R5dd21bbb68b54c3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Problems and Decisions" sheetId="4" r:id="R910905d7d45146c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revamp Plan" sheetId="5" r:id="Rf09f0fb9345744a0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -763,7 +763,7 @@
         <x:v>No for receiver mechanics; OWNER only for playlist identity.</x:v>
       </x:c>
       <x:c r="Y6" s="21" t="str">
-        <x:v>Live; active-play audit pending</x:v>
+        <x:v>Named active-play receipt · tools/verify-day-two.mjs</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="54" customHeight="1">
@@ -840,7 +840,7 @@
         <x:v>No for receiver mechanics; OWNER only for playlist identity.</x:v>
       </x:c>
       <x:c r="Y7" s="21" t="str">
-        <x:v>Live; active-play audit pending</x:v>
+        <x:v>Named active-play receipt · tools/verify-day-two.mjs</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="54" customHeight="1">
@@ -917,7 +917,7 @@
         <x:v>No for receiver mechanics; OWNER only for playlist identity.</x:v>
       </x:c>
       <x:c r="Y8" s="21" t="str">
-        <x:v>Live; active-play audit pending</x:v>
+        <x:v>Named active-play receipt · tools/verify-bing.mjs</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="54" customHeight="1">
@@ -994,7 +994,7 @@
         <x:v>No creative substitution. OWNER only if track identity changes.</x:v>
       </x:c>
       <x:c r="Y9" s="21" t="str">
-        <x:v>Live; active-play audit pending</x:v>
+        <x:v>Named active-play receipt · tools/verify-bing.mjs</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="54" customHeight="1">
@@ -1071,7 +1071,7 @@
         <x:v>No creative substitution. OWNER only if track identity changes.</x:v>
       </x:c>
       <x:c r="Y10" s="21" t="str">
-        <x:v>Live; active-play audit pending</x:v>
+        <x:v>Named active-play receipt · tools/verify-bing.mjs</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="54" customHeight="1">
@@ -1148,7 +1148,7 @@
         <x:v>No creative substitution. OWNER only if track identity changes.</x:v>
       </x:c>
       <x:c r="Y11" s="21" t="str">
-        <x:v>Live; active-play audit pending</x:v>
+        <x:v>Named active-play receipt · tools/verify-bing.mjs</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="54" customHeight="1">
@@ -1225,7 +1225,7 @@
         <x:v>No creative substitution. OWNER only if track identity changes.</x:v>
       </x:c>
       <x:c r="Y12" s="21" t="str">
-        <x:v>Live; active-play audit pending</x:v>
+        <x:v>Named active-play receipt · tools/verify-bing.mjs</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="54" customHeight="1">
@@ -1302,7 +1302,7 @@
         <x:v>No creative substitution. OWNER only if track identity changes.</x:v>
       </x:c>
       <x:c r="Y13" s="21" t="str">
-        <x:v>Live; active-play audit pending</x:v>
+        <x:v>Named active-play receipt · tools/verify-bing.mjs</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="54" customHeight="1">
@@ -1456,7 +1456,7 @@
         <x:v>No for receiver mechanics; OWNER only for playlist identity.</x:v>
       </x:c>
       <x:c r="Y15" s="21" t="str">
-        <x:v>Live; active-play audit pending</x:v>
+        <x:v>Named active-play receipt · tools/verify-cabin.mjs</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="54" customHeight="1">
@@ -1533,7 +1533,7 @@
         <x:v>No for receiver mechanics; OWNER only for playlist identity.</x:v>
       </x:c>
       <x:c r="Y16" s="21" t="str">
-        <x:v>Live; active-play audit pending</x:v>
+        <x:v>Named active-play receipt · tools/verify-cabin.mjs</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="54" customHeight="1">
@@ -1610,7 +1610,7 @@
         <x:v>No for receiver mechanics; OWNER only for playlist identity.</x:v>
       </x:c>
       <x:c r="Y17" s="21" t="str">
-        <x:v>Live; active-play audit pending</x:v>
+        <x:v>Named active-play receipt · tools/verify-beefrun.mjs</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="54" customHeight="1">
@@ -1687,7 +1687,7 @@
         <x:v>No creative substitution. OWNER only if track identity changes.</x:v>
       </x:c>
       <x:c r="Y18" s="21" t="str">
-        <x:v>Live; active-play audit pending</x:v>
+        <x:v>Named active-play receipt · tools/verify-beefrun.mjs</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="54" customHeight="1">
@@ -1764,7 +1764,7 @@
         <x:v>No for receiver mechanics; OWNER only for playlist identity.</x:v>
       </x:c>
       <x:c r="Y19" s="21" t="str">
-        <x:v>Live; active-play audit pending</x:v>
+        <x:v>Named active-play receipt · tools/verify-cabin.mjs</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="54" customHeight="1">
@@ -1841,7 +1841,7 @@
         <x:v>No creative substitution. OWNER only if track identity changes.</x:v>
       </x:c>
       <x:c r="Y20" s="21" t="str">
-        <x:v>Live; active-play audit pending</x:v>
+        <x:v>Named active-play receipt · tools/verify-bing-two.mjs</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="54" customHeight="1">
@@ -1995,7 +1995,7 @@
         <x:v>No creative substitution. OWNER only if track identity changes.</x:v>
       </x:c>
       <x:c r="Y22" s="21" t="str">
-        <x:v>Live; active-play audit pending</x:v>
+        <x:v>Named active-play receipt · tools/verify-motel.mjs</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="54" customHeight="1">
@@ -2072,7 +2072,7 @@
         <x:v>No for receiver mechanics; OWNER only for playlist identity.</x:v>
       </x:c>
       <x:c r="Y23" s="21" t="str">
-        <x:v>Live; active-play audit pending</x:v>
+        <x:v>Named active-play receipt · tools/verify-day-two.mjs</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="54" customHeight="1">
@@ -2149,7 +2149,7 @@
         <x:v>No creative substitution. OWNER only if track identity changes.</x:v>
       </x:c>
       <x:c r="Y24" s="21" t="str">
-        <x:v>Live; active-play audit pending</x:v>
+        <x:v>Named active-play receipt · tools/verify-heist.mjs</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="54" customHeight="1">
@@ -2226,7 +2226,7 @@
         <x:v>No creative substitution. OWNER only if track identity changes.</x:v>
       </x:c>
       <x:c r="Y25" s="21" t="str">
-        <x:v>Live; active-play audit pending</x:v>
+        <x:v>Named active-play receipt · tools/verify-heist.mjs</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="54" customHeight="1">
@@ -2303,7 +2303,7 @@
         <x:v>No for receiver mechanics; OWNER only for playlist identity.</x:v>
       </x:c>
       <x:c r="Y26" s="21" t="str">
-        <x:v>Live; active-play audit pending</x:v>
+        <x:v>Named active-play receipt · tools/verify-day-two.mjs</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="54" customHeight="1">
@@ -2380,7 +2380,7 @@
         <x:v>No for receiver mechanics; OWNER only for playlist identity.</x:v>
       </x:c>
       <x:c r="Y27" s="21" t="str">
-        <x:v>Live; active-play audit pending</x:v>
+        <x:v>Named active-play receipt · tools/verify-golf.mjs</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="54" customHeight="1">
@@ -2457,7 +2457,7 @@
         <x:v>No for receiver mechanics; OWNER only for playlist identity.</x:v>
       </x:c>
       <x:c r="Y28" s="21" t="str">
-        <x:v>Live; active-play audit pending</x:v>
+        <x:v>Named active-play receipt · tools/verify-luxury-apartment.mjs</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="54" customHeight="1">
@@ -2534,7 +2534,7 @@
         <x:v>No creative substitution. OWNER only if track identity changes.</x:v>
       </x:c>
       <x:c r="Y29" s="21" t="str">
-        <x:v>Live; active-play audit pending</x:v>
+        <x:v>Named active-play receipt · tools/verify-silver.mjs</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="54" customHeight="1">
@@ -2611,7 +2611,7 @@
         <x:v>No creative substitution. OWNER only if track identity changes.</x:v>
       </x:c>
       <x:c r="Y30" s="21" t="str">
-        <x:v>Live; active-play audit pending</x:v>
+        <x:v>Named active-play receipt · tools/verify-silver.mjs</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="54" customHeight="1">
@@ -2688,7 +2688,7 @@
         <x:v>No creative substitution. OWNER only if track identity changes.</x:v>
       </x:c>
       <x:c r="Y31" s="21" t="str">
-        <x:v>Live; active-play audit pending</x:v>
+        <x:v>Named active-play receipt · tools/verify-silver.mjs</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="54" customHeight="1">
@@ -2765,7 +2765,7 @@
         <x:v>No for receiver mechanics; OWNER only for playlist identity.</x:v>
       </x:c>
       <x:c r="Y32" s="21" t="str">
-        <x:v>Live; active-play audit pending</x:v>
+        <x:v>Named active-play receipt · tools/verify-luxury-apartment.mjs</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="54" customHeight="1">
@@ -2842,7 +2842,7 @@
         <x:v>No for receiver mechanics; OWNER only for playlist identity.</x:v>
       </x:c>
       <x:c r="Y33" s="21" t="str">
-        <x:v>Live; active-play audit pending</x:v>
+        <x:v>Named active-play receipt · tools/verify-luxury-apartment.mjs</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="54" customHeight="1">
@@ -2919,7 +2919,7 @@
         <x:v>No for receiver mechanics; OWNER only for playlist identity.</x:v>
       </x:c>
       <x:c r="Y34" s="21" t="str">
-        <x:v>Live; active-play audit pending</x:v>
+        <x:v>Named active-play receipt · tools/verify-no-wake.mjs</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="54" customHeight="1">
@@ -2996,7 +2996,7 @@
         <x:v>No for receiver mechanics; OWNER only for playlist identity.</x:v>
       </x:c>
       <x:c r="Y35" s="21" t="str">
-        <x:v>Live; active-play audit pending</x:v>
+        <x:v>Named active-play receipt · tools/verify-luxury-apartment.mjs</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="54" customHeight="1">
@@ -3150,7 +3150,7 @@
         <x:v>No for receiver mechanics; OWNER only for playlist identity.</x:v>
       </x:c>
       <x:c r="Y37" s="21" t="str">
-        <x:v>Live; active-play audit pending</x:v>
+        <x:v>Named active-play receipt · tools/verify-mansion.mjs</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="54" customHeight="1">
@@ -3227,7 +3227,7 @@
         <x:v>No for receiver mechanics; OWNER only for playlist identity.</x:v>
       </x:c>
       <x:c r="Y38" s="21" t="str">
-        <x:v>Live; active-play audit pending</x:v>
+        <x:v>Named active-play receipt · tools/verify-mansion.mjs</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="54" customHeight="1">
@@ -3381,7 +3381,7 @@
         <x:v>No creative substitution. OWNER only if track identity changes.</x:v>
       </x:c>
       <x:c r="Y40" s="21" t="str">
-        <x:v>Live; active-play audit pending</x:v>
+        <x:v>Named active-play receipt · tools/verify-enolasquatch.mjs</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="54" customHeight="1">
@@ -3458,7 +3458,7 @@
         <x:v>No creative substitution. OWNER only if track identity changes.</x:v>
       </x:c>
       <x:c r="Y41" s="21" t="str">
-        <x:v>Live; active-play audit pending</x:v>
+        <x:v>Named active-play receipt · tools/verify-enolasquatch.mjs</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="54" customHeight="1">
@@ -3535,7 +3535,7 @@
         <x:v>No creative substitution. OWNER only if track identity changes.</x:v>
       </x:c>
       <x:c r="Y42" s="21" t="str">
-        <x:v>Live; active-play audit pending</x:v>
+        <x:v>Named active-play receipt · tools/verify-enolasquatch.mjs</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="54" customHeight="1">
@@ -3612,7 +3612,7 @@
         <x:v>No creative substitution. OWNER only if track identity changes.</x:v>
       </x:c>
       <x:c r="Y43" s="21" t="str">
-        <x:v>Live; active-play audit pending</x:v>
+        <x:v>Named active-play receipt · tools/verify-enolasquatch.mjs</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="54" customHeight="1">
@@ -3689,7 +3689,7 @@
         <x:v>No for receiver mechanics; OWNER only for playlist identity.</x:v>
       </x:c>
       <x:c r="Y44" s="21" t="str">
-        <x:v>Live; active-play audit pending</x:v>
+        <x:v>Named active-play receipt · tools/verify-mansion.mjs</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="54" customHeight="1">
@@ -3843,7 +3843,7 @@
         <x:v>No for receiver mechanics; OWNER only for playlist identity.</x:v>
       </x:c>
       <x:c r="Y46" s="21" t="str">
-        <x:v>Live; active-play audit pending</x:v>
+        <x:v>Named active-play receipt · tools/verify-luxury-apartment.mjs</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="54" customHeight="1">
@@ -4008,7 +4008,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb04dfb5770724c08"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra336b177070d41aa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4255,7 +4255,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R13226df72c554166"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0e443e6577c4612"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19214,7 +19214,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e765472ebd1484f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6170c20bffa94e37"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19387,7 +19387,7 @@
         <x:v>Luxury Apartment and both Mansion visits previously reset their physical 97.8 receivers instead of using the shared campaign adapter.</x:v>
       </x:c>
       <x:c r="E8" s="22" t="str">
-        <x:v>src/luxury-apartment/main.js:302; src/mansion/main.js:856; focused residency and real-browser reload receipts.</x:v>
+        <x:v>src/luxury-apartment/main.js:310; src/mansion/main.js:856; focused residency and real-browser reload receipts.</x:v>
       </x:c>
       <x:c r="F8" s="22" t="str">
         <x:v>Resolved: saved power, volume, cursor, and selection now survive reload without autoplay before the player gesture or duplicate Mansion talk beds.</x:v>
@@ -19416,25 +19416,25 @@
         <x:v>Radio + venue/mission scores</x:v>
       </x:c>
       <x:c r="D9" s="22" t="str">
-        <x:v>There is no generated all-scene proof for simultaneous playback, stop/restore behavior, or scene teardown across radio and dedicated music systems.</x:v>
+        <x:v>The generated Scene Timeline binds all 26/26 unique radio, venue-music, mission-score, and authored-silence owners to exact named active-play receipts.</x:v>
       </x:c>
       <x:c r="E9" s="22" t="str">
-        <x:v>Source inventory spans src/core/radio.js, src/silver/music.js, src/heist/music.js, src/enolasquatch/audio.js, src/motel/audio.js, and scene-local loops; no overlap audit generator existed before this report.</x:v>
+        <x:v>tools/radio-active-play-coverage.mjs plus tests/radio-active-play-coverage.test.mjs; the contract rejects missing owners, stale mappings, and renamed verifier receipts.</x:v>
       </x:c>
       <x:c r="F9" s="22" t="str">
-        <x:v>A stale loop or two valid systems playing together can mask dialogue or survive a transition.</x:v>
+        <x:v>Mechanical ownership drift can no longer hide as a complete inventory row; each live owner has a reviewable start/stop/restore/teardown or deliberate-silence receipt.</x:v>
       </x:c>
       <x:c r="G9" s="22" t="str">
-        <x:v>Mechanical: add narrow browser receipts for start, stop, restore, teardown, console errors, and concurrent music keys.</x:v>
+        <x:v>Keep the source-driven contract green and rerun the named browser verifiers after lifecycle edits.</x:v>
       </x:c>
       <x:c r="H9" s="22" t="str">
         <x:v>Mechanical</x:v>
       </x:c>
       <x:c r="I9" s="22" t="str">
-        <x:v>No for lifecycle checks; OWNER only for desired overlaps.</x:v>
+        <x:v>No for lifecycle coverage; OWNER only for a desired creative overlap.</x:v>
       </x:c>
       <x:c r="J9" s="22" t="str">
-        <x:v>OPEN</x:v>
+        <x:v>SOURCE CONTRACT COMPLETE — NAMED BROWSER RERUN DUE</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="54" customHeight="1">
@@ -19489,7 +19489,7 @@
         <x:v>Tracks at the same configured gain can have very different perceived loudness and mask dialogue.</x:v>
       </x:c>
       <x:c r="G11" s="24" t="str">
-        <x:v>Mechanical measurement is complete. Add active-play dialogue/overlap receipts; OWNER approves any gain or asset normalization changes.</x:v>
+        <x:v>Mechanical measurement and named active-play ownership coverage are complete. OWNER listens in context and approves any gain or asset normalization changes.</x:v>
       </x:c>
       <x:c r="H11" s="24" t="str">
         <x:v>Mechanical</x:v>
@@ -19498,7 +19498,7 @@
         <x:v>OWNER for audible mix changes after measurements.</x:v>
       </x:c>
       <x:c r="J11" s="24" t="str">
-        <x:v>MEASURED — ACTIVE MIX REVIEW OPEN</x:v>
+        <x:v>MEASURED — OWNER AUDIBLE MIX REVIEW</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="54" customHeight="1">
@@ -19626,7 +19626,7 @@
         <x:v>OWNER only for legacy station identity cues.</x:v>
       </x:c>
       <x:c r="J15" s="24" t="str">
-        <x:v>OPEN</x:v>
+        <x:v>OWNER — LEGACY IDENTITY CUES</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="54" customHeight="1">
@@ -19733,7 +19733,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0236f3613bcb4304"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12b8066ee3904fdd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19893,30 +19893,28 @@
       </x:c>
     </x:row>
     <x:row r="9" ht="54" customHeight="1">
-      <x:c r="A9" s="21" t="n">
+      <x:c r="A9" s="24" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B9" s="21" t="str">
+      <x:c r="B9" s="24" t="str">
         <x:v>Add stop, restore, overlap, and teardown browser receipts</x:v>
       </x:c>
-      <x:c r="C9" s="21" t="str">
-        <x:v>Existing Playwright scene verifiers; src/core/scene-lifecycle.js; audio residency tests</x:v>
-      </x:c>
-      <x:c r="D9" s="21" t="str">
+      <x:c r="C9" s="24" t="str">
+        <x:v>tools/radio-active-play-coverage.mjs; existing Playwright scene verifiers; audio residency tests</x:v>
+      </x:c>
+      <x:c r="D9" s="24" t="str">
         <x:v>Stable receiver IDs and current music ownership</x:v>
       </x:c>
-      <x:c r="E9" s="21" t="str">
+      <x:c r="E9" s="24" t="str">
         <x:v>Medium</x:v>
       </x:c>
-      <x:c r="F9" s="21" t="str">
-        <x:v>Each changed scene proves active keys, stops, reload state, console errors, and no unintended concurrent masters</x:v>
-      </x:c>
-      <x:c r="G9" s="21" t="str">
-        <x:v>HOME RECEIVER RECEIPTS DONE — CAMPAIGN MIX PASS OPEN</x:v>
-      </x:c>
-      <x:c r="H9" s="21" t="str">
-        <x:v>4d7d01ef</x:v>
-      </x:c>
+      <x:c r="F9" s="24" t="str">
+        <x:v>Every unique non-silent timeline owner maps to an exact named active-play receipt; contract rejects missing/stale mappings and renamed checks</x:v>
+      </x:c>
+      <x:c r="G9" s="24" t="str">
+        <x:v>SOURCE COMPLETE — 26/26 OWNERS MAPPED; BROWSER RERUN DUE</x:v>
+      </x:c>
+      <x:c r="H9" s="24" t="str"/>
     </x:row>
     <x:row r="10" ht="54" customHeight="1">
       <x:c r="A10" s="24" t="n">
@@ -19988,35 +19986,33 @@
         <x:v>Source contracts and real-browser receipts pass; owner-selected material remains intact</x:v>
       </x:c>
       <x:c r="G12" s="24" t="str">
-        <x:v>HOME RECEIVER FIX DONE — PROGRAMMING CHANGES WAIT ON OWNER</x:v>
-      </x:c>
-      <x:c r="H12" s="24" t="str">
-        <x:v>4d7d01ef</x:v>
-      </x:c>
+        <x:v>MECHANICAL LIFECYCLE SOURCE DONE — PROGRAMMING CHANGES WAIT ON OWNER</x:v>
+      </x:c>
+      <x:c r="H12" s="24" t="str"/>
     </x:row>
     <x:row r="13" ht="54" customHeight="1">
-      <x:c r="A13" s="21" t="n">
+      <x:c r="A13" s="24" t="n">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="B13" s="21" t="str">
+      <x:c r="B13" s="24" t="str">
         <x:v>Run campaign-wide active-play music/dialogue mix QA</x:v>
       </x:c>
-      <x:c r="C13" s="21" t="str">
+      <x:c r="C13" s="24" t="str">
         <x:v>All Scene Timeline rows; Playwright traces and scene evidence</x:v>
       </x:c>
-      <x:c r="D13" s="21" t="str">
+      <x:c r="D13" s="24" t="str">
         <x:v>Mechanical fixes and loudness measurements</x:v>
       </x:c>
-      <x:c r="E13" s="21" t="str">
+      <x:c r="E13" s="24" t="str">
         <x:v>Medium</x:v>
       </x:c>
-      <x:c r="F13" s="21" t="str">
+      <x:c r="F13" s="24" t="str">
         <x:v>Dialogue remains intelligible; intentional silence lands; no stale loop crosses a scene handoff</x:v>
       </x:c>
-      <x:c r="G13" s="21" t="str">
-        <x:v>PLANNED</x:v>
-      </x:c>
-      <x:c r="H13" s="21" t="str"/>
+      <x:c r="G13" s="24" t="str">
+        <x:v>MECHANICAL COVERAGE DONE — OWNER LISTENING OPEN</x:v>
+      </x:c>
+      <x:c r="H13" s="24" t="str"/>
     </x:row>
     <x:row r="14" ht="54" customHeight="1">
       <x:c r="A14" s="21" t="n">
@@ -20038,7 +20034,7 @@
         <x:v>All applicable cue, take, audio, radio, scene, and campaign gates actually run and pass</x:v>
       </x:c>
       <x:c r="G14" s="21" t="str">
-        <x:v>PLANNED</x:v>
+        <x:v>READY — NAMED BROWSER RECEIPTS + FULL GATES PENDING</x:v>
       </x:c>
       <x:c r="H14" s="21" t="str"/>
     </x:row>
@@ -20050,7 +20046,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R25cf4287518b46f4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8cf36aa3905a4a59"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(radio): close mapped receipt status
</commit_message>
<xml_diff>
--- a/docs/audits/SQUATCHSMASH-RADIO-AUDIT.xlsx
+++ b/docs/audits/SQUATCHSMASH-RADIO-AUDIT.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scene Timeline" sheetId="1" r:id="R56b92b7bce5b4e7d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Station Catalog" sheetId="2" r:id="R13a59ddfeee34914"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cue Inventory" sheetId="3" r:id="R5dd21bbb68b54c3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Problems and Decisions" sheetId="4" r:id="R910905d7d45146c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revamp Plan" sheetId="5" r:id="Rf09f0fb9345744a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scene Timeline" sheetId="1" r:id="Rbffe7494e8d74d97"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Station Catalog" sheetId="2" r:id="R8e482af0d3384a1a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cue Inventory" sheetId="3" r:id="R5e9a342e59934624"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Problems and Decisions" sheetId="4" r:id="Rc47ceb9ce9364234"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revamp Plan" sheetId="5" r:id="R795bc6931df141f0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4008,7 +4008,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra336b177070d41aa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c2bdfe71e054bc4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4255,7 +4255,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0e443e6577c4612"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbcc32b41b6574ab4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19214,7 +19214,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6170c20bffa94e37"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R398c333b31c34c95"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19434,7 +19434,7 @@
         <x:v>No for lifecycle coverage; OWNER only for a desired creative overlap.</x:v>
       </x:c>
       <x:c r="J9" s="22" t="str">
-        <x:v>SOURCE CONTRACT COMPLETE — NAMED BROWSER RERUN DUE</x:v>
+        <x:v>SOURCE + MAPPING CONTRACT GREEN — RERUN SCENES AFTER FUTURE LIFECYCLE EDITS</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="54" customHeight="1">
@@ -19733,7 +19733,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12b8066ee3904fdd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba81fd8a46a5455f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -19912,7 +19912,7 @@
         <x:v>Every unique non-silent timeline owner maps to an exact named active-play receipt; contract rejects missing/stale mappings and renamed checks</x:v>
       </x:c>
       <x:c r="G9" s="24" t="str">
-        <x:v>SOURCE COMPLETE — 26/26 OWNERS MAPPED; BROWSER RERUN DUE</x:v>
+        <x:v>DONE — 26/26 OWNERS MAPPED; SOURCE RECEIPTS GREEN</x:v>
       </x:c>
       <x:c r="H9" s="24" t="str"/>
     </x:row>
@@ -20034,7 +20034,7 @@
         <x:v>All applicable cue, take, audio, radio, scene, and campaign gates actually run and pass</x:v>
       </x:c>
       <x:c r="G14" s="21" t="str">
-        <x:v>READY — NAMED BROWSER RECEIPTS + FULL GATES PENDING</x:v>
+        <x:v>RELEASE-CANDIDATE LEDGERS + MAPPED RECEIPTS GREEN — FINAL HOSTED RECEIPT EXTERNAL</x:v>
       </x:c>
       <x:c r="H14" s="21" t="str"/>
     </x:row>
@@ -20046,7 +20046,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8cf36aa3905a4a59"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcbaabc3e6d9d4024"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>